<commit_message>
Fix missing feed class
</commit_message>
<xml_diff>
--- a/data/raw_data/feed_profiles_and_composition.xlsx
+++ b/data/raw_data/feed_profiles_and_composition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\climate_risks_to_fed_mariculture\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15AB620-1043-41B8-A22F-996403FA178E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D15D74-3C5D-4EFF-8CDA-C0E2B84919F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7572" yWindow="1344" windowWidth="26880" windowHeight="13908" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11280" yWindow="1044" windowWidth="27396" windowHeight="13908" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="feed_formulations" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="229">
   <si>
     <t>ingredient</t>
   </si>
@@ -446,9 +446,6 @@
     <t>atlantic_salmon</t>
   </si>
   <si>
-    <t>Democratic People's Republic of Korea</t>
-  </si>
-  <si>
     <t>Iran</t>
   </si>
   <si>
@@ -599,9 +596,6 @@
     <t>Aas, T. S. et al. (2022). Utilization of feed resources in the production of Atlantic salmon (Salmo salar) in Norway: An update for 2020. Aquaculture Reports, 26, 101316. https://doi.org/10.1016/j.aqrep.2022.101316</t>
   </si>
   <si>
-    <t>WIP</t>
-  </si>
-  <si>
     <t>rainbow_trout-norway</t>
   </si>
   <si>
@@ -656,9 +650,6 @@
     <t>cellulose</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>Petereit, J., Hoerterer, C., Bischoff-Lang, A. A., Conceição, L. E. C., Pereira, G., Johansen, J., Pastres, R., &amp; Buck, B. H. (2022). Adult European Seabass (Dicentrarchus labrax) Perform Well on Alternative Circular-Economy-Driven Feed Formulations. Sustainability, 14(12), 7279. https://doi.org/10.3390/su14127279</t>
   </si>
   <si>
@@ -743,13 +734,16 @@
     <t>Novriadi, R., Herawati, V. E., Prayitno, S. B., Windarto, S., &amp; Tan, R. (2024). Evaluation of distiller’s dried grains with solubles in diets for Pacific white shrimp, Litopenaeus vannamei, reared under pond conditions. Journal of the World Aquaculture Society, 55(1), 62–76. https://doi.org/10.1111/jwas.13033</t>
   </si>
   <si>
+    <t>wip</t>
+  </si>
+  <si>
+    <t>Reunion</t>
+  </si>
+  <si>
     <t>y</t>
   </si>
   <si>
-    <t>wip</t>
-  </si>
-  <si>
-    <t>Reunion</t>
+    <t>Democratic People’s Republic of Korea</t>
   </si>
 </sst>
 </file>
@@ -1167,7 +1161,7 @@
         <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -1182,7 +1176,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>1</v>
@@ -1194,7 +1188,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>2</v>
@@ -1206,7 +1200,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>24</v>
@@ -1218,7 +1212,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>23</v>
@@ -1230,7 +1224,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>25</v>
@@ -1242,7 +1236,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
@@ -1353,7 +1347,7 @@
         <v>49</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C16" s="2">
         <v>1.4999999999999999E-2</v>
@@ -1938,7 +1932,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>10</v>
@@ -1950,7 +1944,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>9</v>
@@ -1962,7 +1956,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>1</v>
@@ -1974,7 +1968,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>3</v>
@@ -1986,7 +1980,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>2</v>
@@ -1998,7 +1992,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>21</v>
@@ -2010,7 +2004,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>6</v>
@@ -2022,7 +2016,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>22</v>
@@ -2034,7 +2028,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>23</v>
@@ -2046,7 +2040,7 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>14</v>
@@ -2058,7 +2052,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>5</v>
@@ -2070,7 +2064,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>15</v>
@@ -2082,10 +2076,10 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C77" s="2">
         <v>3.7600000000000001E-2</v>
@@ -2094,7 +2088,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>9</v>
@@ -2106,7 +2100,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>1</v>
@@ -2118,7 +2112,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>2</v>
@@ -2130,7 +2124,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>34</v>
@@ -2142,7 +2136,7 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>24</v>
@@ -2154,7 +2148,7 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>22</v>
@@ -2166,7 +2160,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>23</v>
@@ -2178,7 +2172,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>12</v>
@@ -2190,7 +2184,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>25</v>
@@ -2202,7 +2196,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>5</v>
@@ -2330,10 +2324,10 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C96" s="2">
         <v>1.4999999999999999E-2</v>
@@ -2342,10 +2336,10 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C97" s="2">
         <v>0.13</v>
@@ -2354,7 +2348,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>1</v>
@@ -2366,10 +2360,10 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C99" s="2">
         <v>0.08</v>
@@ -2378,7 +2372,7 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>28</v>
@@ -2390,7 +2384,7 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>23</v>
@@ -2402,7 +2396,7 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>12</v>
@@ -2414,10 +2408,10 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B103" s="2" t="s">
         <v>206</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>209</v>
       </c>
       <c r="C103" s="2">
         <v>0.15</v>
@@ -2426,7 +2420,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>15</v>
@@ -2453,7 +2447,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>46</v>
@@ -2465,7 +2459,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>10</v>
@@ -2477,7 +2471,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>9</v>
@@ -2489,7 +2483,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>47</v>
@@ -2501,7 +2495,7 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>1</v>
@@ -2511,12 +2505,12 @@
         <v>7.8947368421052627E-2</v>
       </c>
       <c r="D112" s="12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>3</v>
@@ -2526,12 +2520,12 @@
         <v>7.1052631578947367E-2</v>
       </c>
       <c r="D113" s="12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>2</v>
@@ -2541,12 +2535,12 @@
         <v>3.428571428571428E-2</v>
       </c>
       <c r="D114" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>4</v>
@@ -2556,12 +2550,12 @@
         <v>2.571428571428571E-2</v>
       </c>
       <c r="D115" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>34</v>
@@ -2573,10 +2567,10 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C117" s="2">
         <v>0.03</v>
@@ -2585,7 +2579,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>22</v>
@@ -2597,7 +2591,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>14</v>
@@ -2609,7 +2603,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>5</v>
@@ -2621,7 +2615,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>15</v>
@@ -2633,7 +2627,7 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>10</v>
@@ -2645,7 +2639,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>13</v>
@@ -2657,7 +2651,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>17</v>
@@ -2669,7 +2663,7 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>1</v>
@@ -2681,7 +2675,7 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>3</v>
@@ -2693,7 +2687,7 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>2</v>
@@ -2705,7 +2699,7 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>4</v>
@@ -2717,7 +2711,7 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>16</v>
@@ -2729,7 +2723,7 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>11</v>
@@ -2741,7 +2735,7 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>20</v>
@@ -2753,7 +2747,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>18</v>
@@ -2765,7 +2759,7 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>12</v>
@@ -2777,7 +2771,7 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>14</v>
@@ -2789,7 +2783,7 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>19</v>
@@ -2801,7 +2795,7 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>5</v>
@@ -2813,7 +2807,7 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>15</v>
@@ -2825,7 +2819,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>9</v>
@@ -2837,7 +2831,7 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>47</v>
@@ -2849,7 +2843,7 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>1</v>
@@ -2859,12 +2853,12 @@
         <v>0.15789473684210525</v>
       </c>
       <c r="D140" s="12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>3</v>
@@ -2874,12 +2868,12 @@
         <v>0.14210526315789473</v>
       </c>
       <c r="D141" s="12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>2</v>
@@ -2889,12 +2883,12 @@
         <v>5.1428571428571421E-2</v>
       </c>
       <c r="D142" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>4</v>
@@ -2904,12 +2898,12 @@
         <v>3.8571428571428562E-2</v>
       </c>
       <c r="D143" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>34</v>
@@ -2921,10 +2915,10 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C145" s="2">
         <v>0.04</v>
@@ -2933,7 +2927,7 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>22</v>
@@ -2945,7 +2939,7 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>23</v>
@@ -2957,7 +2951,7 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>12</v>
@@ -2969,7 +2963,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>5</v>
@@ -2981,10 +2975,10 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C150" s="2">
         <v>7.1999999999999995E-2</v>
@@ -2993,7 +2987,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>1</v>
@@ -3005,7 +2999,7 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>2</v>
@@ -3017,7 +3011,7 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>34</v>
@@ -3030,7 +3024,7 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B154" s="2" t="s">
         <v>23</v>
@@ -3042,7 +3036,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>14</v>
@@ -3054,7 +3048,7 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>5</v>
@@ -3066,7 +3060,7 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>1</v>
@@ -3078,7 +3072,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>2</v>
@@ -3090,7 +3084,7 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>26</v>
@@ -3102,7 +3096,7 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>8</v>
@@ -3114,7 +3108,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>12</v>
@@ -3126,7 +3120,7 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>14</v>
@@ -3138,7 +3132,7 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>5</v>
@@ -3150,7 +3144,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>15</v>
@@ -3172,7 +3166,7 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>23</v>
@@ -3184,7 +3178,7 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>22</v>
@@ -3195,7 +3189,7 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>1</v>
@@ -3206,7 +3200,7 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>25</v>
@@ -3217,7 +3211,7 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>5</v>
@@ -3228,7 +3222,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>2</v>
@@ -3239,7 +3233,7 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>34</v>
@@ -3251,7 +3245,7 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>1</v>
@@ -3262,10 +3256,10 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C175">
         <v>0.12</v>
@@ -3273,10 +3267,10 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C176">
         <v>0.1474</v>
@@ -3284,7 +3278,7 @@
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>23</v>
@@ -3295,10 +3289,10 @@
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B178" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="B178" s="2" t="s">
-        <v>222</v>
       </c>
       <c r="C178">
         <v>1.15E-2</v>
@@ -3306,10 +3300,10 @@
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C179">
         <v>0.02</v>
@@ -3317,7 +3311,7 @@
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B180" s="2" t="s">
         <v>34</v>
@@ -3328,10 +3322,10 @@
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B181" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C181">
         <v>0.05</v>
@@ -3339,7 +3333,7 @@
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B182" t="s">
         <v>1</v>
@@ -3350,7 +3344,7 @@
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B183" t="s">
         <v>3</v>
@@ -3361,7 +3355,7 @@
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B184" t="s">
         <v>34</v>
@@ -3372,7 +3366,7 @@
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B185" t="s">
         <v>23</v>
@@ -3383,7 +3377,7 @@
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B186" t="s">
         <v>12</v>
@@ -3394,7 +3388,7 @@
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B187" t="s">
         <v>5</v>
@@ -3405,7 +3399,7 @@
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B188" t="s">
         <v>1</v>
@@ -3416,7 +3410,7 @@
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B189" t="s">
         <v>2</v>
@@ -3427,7 +3421,7 @@
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B190" t="s">
         <v>34</v>
@@ -3438,7 +3432,7 @@
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B191" t="s">
         <v>23</v>
@@ -3449,7 +3443,7 @@
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B192" t="s">
         <v>5</v>
@@ -4395,49 +4389,49 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>174</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C2" s="8">
         <v>223</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>94</v>
@@ -4446,7 +4440,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E3" s="11"/>
       <c r="F3" s="8"/>
@@ -4454,7 +4448,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>83</v>
@@ -4463,7 +4457,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E4" s="11"/>
       <c r="F4" s="8"/>
@@ -4471,7 +4465,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>57</v>
@@ -4480,7 +4474,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="8"/>
@@ -4491,16 +4485,16 @@
         <v>128</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C6" s="8">
         <v>159</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
@@ -4510,13 +4504,13 @@
         <v>128</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C7" s="8">
         <v>50</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="8"/>
@@ -4533,7 +4527,7 @@
         <v>21</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="8"/>
@@ -4550,13 +4544,13 @@
         <v>1494</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>180</v>
+        <v>225</v>
       </c>
       <c r="G9" s="8"/>
     </row>
@@ -4565,20 +4559,20 @@
         <v>128</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>129</v>
+        <v>228</v>
       </c>
       <c r="C10" s="8">
         <v>1</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="8" t="s">
-        <v>180</v>
+        <v>225</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
@@ -4586,20 +4580,18 @@
         <v>128</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C11" s="8">
         <v>863</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>199</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="F11" s="8"/>
       <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -4607,18 +4599,16 @@
         <v>128</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12" s="8">
         <v>22</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E12" s="11"/>
-      <c r="F12" s="8" t="s">
-        <v>199</v>
-      </c>
+      <c r="F12" s="8"/>
       <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -4626,18 +4616,16 @@
         <v>128</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C13" s="8">
         <v>16</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E13" s="11"/>
-      <c r="F13" s="8" t="s">
-        <v>199</v>
-      </c>
+      <c r="F13" s="8"/>
       <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -4645,18 +4633,16 @@
         <v>128</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C14" s="8">
         <v>9</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E14" s="11"/>
-      <c r="F14" s="8" t="s">
-        <v>199</v>
-      </c>
+      <c r="F14" s="8"/>
       <c r="G14" s="8"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -4664,18 +4650,16 @@
         <v>128</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C15" s="8">
         <v>5</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E15" s="11"/>
-      <c r="F15" s="8" t="s">
-        <v>199</v>
-      </c>
+      <c r="F15" s="8"/>
       <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
@@ -4683,7 +4667,7 @@
         <v>128</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C16" s="8">
         <v>212</v>
@@ -4692,7 +4676,7 @@
         <v>127</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -4702,7 +4686,7 @@
         <v>128</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C17" s="8">
         <v>63</v>
@@ -4770,7 +4754,7 @@
         <v>119</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C21" s="8">
         <v>161</v>
@@ -4785,7 +4769,7 @@
         <v>119</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C22" s="8">
         <v>16</v>
@@ -4860,7 +4844,7 @@
         <v>119</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C27" s="8">
         <v>4</v>
@@ -5166,10 +5150,10 @@
         <v>259</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -5185,7 +5169,7 @@
         <v>60</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E48" s="11"/>
       <c r="F48" s="8"/>
@@ -5202,7 +5186,7 @@
         <v>34</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E49" s="11"/>
       <c r="F49" s="8"/>
@@ -5213,13 +5197,13 @@
         <v>118</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C50" s="8">
         <v>28</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E50" s="11"/>
       <c r="F50" s="8"/>
@@ -5236,7 +5220,7 @@
         <v>22</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E51" s="11"/>
       <c r="F51" s="8"/>
@@ -5247,13 +5231,13 @@
         <v>118</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C52" s="8">
         <v>19</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E52" s="11"/>
       <c r="F52" s="8"/>
@@ -5270,7 +5254,7 @@
         <v>16</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E53" s="11"/>
       <c r="F53" s="8"/>
@@ -5287,7 +5271,7 @@
         <v>9</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E54" s="11"/>
       <c r="F54" s="8"/>
@@ -5304,7 +5288,7 @@
         <v>4</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E55" s="11"/>
       <c r="F55" s="8"/>
@@ -5321,7 +5305,7 @@
         <v>3</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E56" s="11"/>
       <c r="F56" s="8"/>
@@ -5338,7 +5322,7 @@
         <v>2</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E57" s="11"/>
       <c r="F57" s="8"/>
@@ -5349,13 +5333,13 @@
         <v>118</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C58" s="8">
         <v>2</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E58" s="11"/>
       <c r="F58" s="8"/>
@@ -5372,7 +5356,7 @@
         <v>2</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E59" s="11"/>
       <c r="F59" s="8"/>
@@ -5389,7 +5373,7 @@
         <v>2</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E60" s="11"/>
       <c r="F60" s="8"/>
@@ -5406,7 +5390,7 @@
         <v>1</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E61" s="11"/>
       <c r="F61" s="8"/>
@@ -5423,7 +5407,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E62" s="11"/>
       <c r="F62" s="8"/>
@@ -5440,7 +5424,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E63" s="11"/>
       <c r="F63" s="8"/>
@@ -5457,7 +5441,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E64" s="11"/>
       <c r="F64" s="8"/>
@@ -5474,7 +5458,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E65" s="11"/>
       <c r="F65" s="8"/>
@@ -5491,7 +5475,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E66" s="11"/>
       <c r="F66" s="8"/>
@@ -5508,7 +5492,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E67" s="11"/>
       <c r="F67" s="8"/>
@@ -5525,7 +5509,7 @@
         <v>1</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E68" s="11"/>
       <c r="F68" s="8"/>
@@ -5542,7 +5526,7 @@
         <v>1</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E69" s="11"/>
       <c r="F69" s="8"/>
@@ -5553,16 +5537,16 @@
         <v>117</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C70" s="8">
         <v>239</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F70" s="8"/>
       <c r="G70" s="8"/>
@@ -5572,13 +5556,13 @@
         <v>117</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C71" s="8">
         <v>4</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E71" s="11"/>
       <c r="F71" s="8"/>
@@ -5595,7 +5579,7 @@
         <v>4</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E72" s="11"/>
       <c r="F72" s="8"/>
@@ -5606,13 +5590,13 @@
         <v>117</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C73" s="8">
         <v>2</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E73" s="11"/>
       <c r="F73" s="8"/>
@@ -5629,7 +5613,7 @@
         <v>1</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E74" s="11"/>
       <c r="F74" s="8"/>
@@ -5646,7 +5630,7 @@
         <v>1</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E75" s="11"/>
       <c r="F75" s="8"/>
@@ -5663,7 +5647,7 @@
         <v>1</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E76" s="11"/>
       <c r="F76" s="8"/>
@@ -5680,7 +5664,7 @@
         <v>1</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E77" s="11"/>
       <c r="F77" s="8"/>
@@ -5691,7 +5675,7 @@
         <v>113</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C78" s="8">
         <v>214</v>
@@ -5721,7 +5705,7 @@
         <v>113</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C80" s="8">
         <v>8</v>
@@ -5736,7 +5720,7 @@
         <v>113</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C81" s="8">
         <v>3</v>
@@ -5781,7 +5765,7 @@
         <v>113</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C84" s="8">
         <v>2</v>
@@ -5931,7 +5915,7 @@
         <v>33</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C94" s="8">
         <v>150</v>
@@ -5946,7 +5930,7 @@
         <v>33</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C95" s="8">
         <v>29</v>
@@ -6066,16 +6050,16 @@
         <v>36</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C103" s="8">
         <v>433</v>
       </c>
       <c r="D103" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E103" s="9" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F103" s="8"/>
       <c r="G103" s="8"/>
@@ -6091,7 +6075,7 @@
         <v>214</v>
       </c>
       <c r="D104" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E104" s="11"/>
       <c r="F104" s="8"/>
@@ -6108,7 +6092,7 @@
         <v>50</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E105" s="11"/>
       <c r="F105" s="8"/>
@@ -6125,7 +6109,7 @@
         <v>31</v>
       </c>
       <c r="D106" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E106" s="11"/>
       <c r="F106" s="8"/>
@@ -6136,13 +6120,13 @@
         <v>36</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C107" s="8">
         <v>6</v>
       </c>
       <c r="D107" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E107" s="11"/>
       <c r="F107" s="8"/>
@@ -6159,7 +6143,7 @@
         <v>1</v>
       </c>
       <c r="D108" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E108" s="11"/>
       <c r="F108" s="8"/>
@@ -6176,7 +6160,7 @@
         <v>1</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E109" s="11"/>
       <c r="F109" s="8"/>
@@ -6193,7 +6177,7 @@
         <v>1</v>
       </c>
       <c r="D110" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E110" s="11"/>
       <c r="F110" s="8"/>
@@ -6210,7 +6194,7 @@
         <v>1</v>
       </c>
       <c r="D111" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E111" s="11"/>
       <c r="F111" s="8"/>
@@ -6227,7 +6211,7 @@
         <v>1</v>
       </c>
       <c r="D112" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E112" s="11"/>
       <c r="F112" s="8"/>
@@ -6244,7 +6228,7 @@
         <v>1</v>
       </c>
       <c r="D113" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E113" s="11"/>
       <c r="F113" s="8"/>
@@ -6261,7 +6245,7 @@
         <v>1</v>
       </c>
       <c r="D114" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E114" s="11"/>
       <c r="F114" s="8"/>
@@ -6278,7 +6262,7 @@
         <v>1</v>
       </c>
       <c r="D115" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E115" s="11"/>
       <c r="F115" s="8"/>
@@ -6295,7 +6279,7 @@
         <v>1</v>
       </c>
       <c r="D116" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E116" s="11"/>
       <c r="F116" s="8"/>
@@ -6312,7 +6296,7 @@
         <v>1</v>
       </c>
       <c r="D117" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E117" s="11"/>
       <c r="F117" s="8"/>
@@ -6329,7 +6313,7 @@
         <v>1</v>
       </c>
       <c r="D118" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E118" s="11"/>
       <c r="F118" s="8"/>
@@ -6346,7 +6330,7 @@
         <v>1</v>
       </c>
       <c r="D119" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E119" s="11"/>
       <c r="F119" s="8"/>
@@ -6357,7 +6341,7 @@
         <v>40</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C120" s="8">
         <v>468</v>
@@ -6372,7 +6356,7 @@
         <v>40</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C121" s="8">
         <v>96</v>
@@ -6387,7 +6371,7 @@
         <v>40</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C122" s="8">
         <v>38</v>
@@ -6417,7 +6401,7 @@
         <v>40</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C124" s="8">
         <v>22</v>
@@ -6432,7 +6416,7 @@
         <v>40</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C125" s="8">
         <v>21</v>
@@ -6462,7 +6446,7 @@
         <v>40</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C127" s="8">
         <v>7</v>
@@ -6477,7 +6461,7 @@
         <v>40</v>
       </c>
       <c r="B128" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C128" s="8">
         <v>2</v>
@@ -6702,7 +6686,7 @@
         <v>37</v>
       </c>
       <c r="B143" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C143" s="8">
         <v>60</v>
@@ -6762,7 +6746,7 @@
         <v>37</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C147" s="8">
         <v>2</v>
@@ -6822,7 +6806,7 @@
         <v>37</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C151" s="8">
         <v>1</v>
@@ -6942,7 +6926,7 @@
         <v>38</v>
       </c>
       <c r="B159" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C159" s="8">
         <v>39</v>
@@ -6957,7 +6941,7 @@
         <v>38</v>
       </c>
       <c r="B160" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C160" s="8">
         <v>3</v>
@@ -6982,23 +6966,25 @@
       <c r="F161" s="8"/>
       <c r="G161" s="8"/>
     </row>
-    <row r="162" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A162" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B162" s="8" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="C162" s="8">
-        <v>334</v>
+        <v>263</v>
       </c>
       <c r="D162" s="8" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
       <c r="E162" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="F162" s="8"/>
+        <v>185</v>
+      </c>
+      <c r="F162" s="8" t="s">
+        <v>227</v>
+      </c>
       <c r="G162" s="8"/>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.25">
@@ -7006,36 +6992,35 @@
         <v>93</v>
       </c>
       <c r="B163" s="8" t="s">
-        <v>97</v>
+        <v>160</v>
       </c>
       <c r="C163" s="8">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="D163" s="8" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
       <c r="E163" s="11"/>
-      <c r="F163" s="8"/>
-      <c r="G163" s="8"/>
-    </row>
-    <row r="164" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="F163" s="8" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B164" s="8" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C164" s="8">
-        <v>263</v>
+        <v>12</v>
       </c>
       <c r="D164" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="E164" s="9" t="s">
-        <v>187</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="E164" s="11"/>
       <c r="F164" s="8" t="s">
-        <v>180</v>
+        <v>227</v>
       </c>
       <c r="G164" s="8"/>
     </row>
@@ -7044,54 +7029,57 @@
         <v>93</v>
       </c>
       <c r="B165" s="8" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="C165" s="8">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="D165" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E165" s="11"/>
       <c r="F165" s="8" t="s">
-        <v>229</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="G165" s="8"/>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B166" s="8" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="C166" s="8">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D166" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E166" s="11"/>
       <c r="F166" s="8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="G166" s="8"/>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A167" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B167" s="8" t="s">
-        <v>149</v>
+        <v>53</v>
       </c>
       <c r="C167" s="8">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="D167" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="E167" s="11"/>
+        <v>180</v>
+      </c>
+      <c r="E167" s="9" t="s">
+        <v>183</v>
+      </c>
       <c r="F167" s="8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="G167" s="8"/>
     </row>
@@ -7100,38 +7088,36 @@
         <v>93</v>
       </c>
       <c r="B168" s="8" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="C168" s="8">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="D168" s="8" t="s">
-        <v>143</v>
+        <v>180</v>
       </c>
       <c r="E168" s="11"/>
       <c r="F168" s="8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="G168" s="8"/>
     </row>
-    <row r="169" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B169" s="8" t="s">
-        <v>53</v>
+        <v>145</v>
       </c>
       <c r="C169" s="8">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D169" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E169" s="9" t="s">
-        <v>185</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="E169" s="11"/>
       <c r="F169" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G169" s="8"/>
     </row>
@@ -7140,17 +7126,17 @@
         <v>93</v>
       </c>
       <c r="B170" s="8" t="s">
-        <v>156</v>
+        <v>138</v>
       </c>
       <c r="C170" s="8">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D170" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E170" s="11"/>
       <c r="F170" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G170" s="8"/>
     </row>
@@ -7159,17 +7145,17 @@
         <v>93</v>
       </c>
       <c r="B171" s="8" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C171" s="8">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="D171" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E171" s="11"/>
       <c r="F171" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G171" s="8"/>
     </row>
@@ -7178,17 +7164,17 @@
         <v>93</v>
       </c>
       <c r="B172" s="8" t="s">
-        <v>139</v>
+        <v>96</v>
       </c>
       <c r="C172" s="8">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D172" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E172" s="11"/>
       <c r="F172" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G172" s="8"/>
     </row>
@@ -7197,17 +7183,17 @@
         <v>93</v>
       </c>
       <c r="B173" s="8" t="s">
-        <v>140</v>
+        <v>95</v>
       </c>
       <c r="C173" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D173" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E173" s="11"/>
       <c r="F173" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G173" s="8"/>
     </row>
@@ -7216,17 +7202,17 @@
         <v>93</v>
       </c>
       <c r="B174" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C174" s="8">
         <v>1</v>
       </c>
       <c r="D174" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E174" s="11"/>
       <c r="F174" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G174" s="8"/>
     </row>
@@ -7235,36 +7221,38 @@
         <v>93</v>
       </c>
       <c r="B175" s="8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C175" s="8">
         <v>1</v>
       </c>
       <c r="D175" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E175" s="11"/>
       <c r="F175" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G175" s="8"/>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B176" s="8" t="s">
-        <v>94</v>
+        <v>126</v>
       </c>
       <c r="C176" s="8">
-        <v>1</v>
+        <v>334</v>
       </c>
       <c r="D176" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E176" s="11"/>
+        <v>168</v>
+      </c>
+      <c r="E176" s="9" t="s">
+        <v>184</v>
+      </c>
       <c r="F176" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="G176" s="8"/>
     </row>
@@ -7273,17 +7261,17 @@
         <v>93</v>
       </c>
       <c r="B177" s="8" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C177" s="8">
         <v>1</v>
       </c>
       <c r="D177" s="8" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="E177" s="11"/>
       <c r="F177" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="G177" s="8"/>
     </row>
@@ -7292,16 +7280,16 @@
         <v>82</v>
       </c>
       <c r="B178" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C178" s="8">
         <v>134</v>
       </c>
       <c r="D178" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E178" s="9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F178" s="8"/>
       <c r="G178" s="8"/>
@@ -7311,13 +7299,13 @@
         <v>82</v>
       </c>
       <c r="B179" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C179" s="8">
         <v>76</v>
       </c>
       <c r="D179" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E179" s="11"/>
       <c r="F179" s="8"/>
@@ -7334,7 +7322,7 @@
         <v>17</v>
       </c>
       <c r="D180" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E180" s="11"/>
       <c r="F180" s="8"/>
@@ -7345,13 +7333,13 @@
         <v>82</v>
       </c>
       <c r="B181" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C181" s="8">
         <v>2</v>
       </c>
       <c r="D181" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E181" s="11"/>
       <c r="F181" s="8"/>
@@ -7368,7 +7356,7 @@
         <v>1</v>
       </c>
       <c r="D182" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E182" s="11"/>
       <c r="F182" s="8"/>
@@ -7385,7 +7373,7 @@
         <v>1</v>
       </c>
       <c r="D183" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E183" s="11"/>
       <c r="F183" s="8"/>
@@ -7402,7 +7390,7 @@
         <v>1</v>
       </c>
       <c r="D184" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E184" s="11"/>
       <c r="F184" s="8"/>
@@ -7419,7 +7407,7 @@
         <v>1</v>
       </c>
       <c r="D185" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E185" s="11"/>
       <c r="F185" s="8"/>
@@ -7436,7 +7424,7 @@
         <v>1</v>
       </c>
       <c r="D186" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E186" s="11"/>
       <c r="F186" s="8"/>
@@ -7453,7 +7441,7 @@
         <v>1</v>
       </c>
       <c r="D187" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E187" s="11"/>
       <c r="F187" s="8"/>
@@ -7470,7 +7458,7 @@
         <v>1</v>
       </c>
       <c r="D188" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E188" s="11"/>
       <c r="F188" s="8"/>
@@ -7487,7 +7475,7 @@
         <v>1</v>
       </c>
       <c r="D189" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E189" s="11"/>
       <c r="F189" s="8"/>
@@ -7504,7 +7492,7 @@
         <v>1</v>
       </c>
       <c r="D190" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E190" s="11"/>
       <c r="F190" s="8"/>
@@ -7521,7 +7509,7 @@
         <v>1</v>
       </c>
       <c r="D191" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E191" s="11"/>
       <c r="F191" s="8"/>
@@ -7538,10 +7526,10 @@
         <v>59</v>
       </c>
       <c r="D192" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E192" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F192" s="8"/>
       <c r="G192" s="8"/>
@@ -7557,7 +7545,7 @@
         <v>40</v>
       </c>
       <c r="D193" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E193" s="11"/>
       <c r="F193" s="8"/>
@@ -7568,13 +7556,13 @@
         <v>82</v>
       </c>
       <c r="B194" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C194" s="8">
         <v>26</v>
       </c>
       <c r="D194" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E194" s="11"/>
       <c r="F194" s="8"/>
@@ -7591,7 +7579,7 @@
         <v>25</v>
       </c>
       <c r="D195" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E195" s="11"/>
       <c r="F195" s="8"/>
@@ -7602,13 +7590,13 @@
         <v>82</v>
       </c>
       <c r="B196" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C196" s="8">
         <v>23</v>
       </c>
       <c r="D196" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E196" s="11"/>
       <c r="F196" s="8"/>
@@ -7625,7 +7613,7 @@
         <v>18</v>
       </c>
       <c r="D197" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E197" s="11"/>
       <c r="F197" s="8"/>
@@ -7642,7 +7630,7 @@
         <v>14</v>
       </c>
       <c r="D198" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E198" s="11"/>
       <c r="F198" s="8"/>
@@ -7653,13 +7641,13 @@
         <v>82</v>
       </c>
       <c r="B199" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C199" s="8">
         <v>14</v>
       </c>
       <c r="D199" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E199" s="11"/>
       <c r="F199" s="8"/>
@@ -7676,7 +7664,7 @@
         <v>10</v>
       </c>
       <c r="D200" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E200" s="11"/>
       <c r="F200" s="8"/>
@@ -7693,7 +7681,7 @@
         <v>9</v>
       </c>
       <c r="D201" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E201" s="11"/>
       <c r="F201" s="8"/>
@@ -7710,7 +7698,7 @@
         <v>3</v>
       </c>
       <c r="D202" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E202" s="11"/>
       <c r="F202" s="8"/>
@@ -7721,13 +7709,13 @@
         <v>82</v>
       </c>
       <c r="B203" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C203" s="8">
         <v>3</v>
       </c>
       <c r="D203" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E203" s="11"/>
       <c r="F203" s="8"/>
@@ -7744,7 +7732,7 @@
         <v>2</v>
       </c>
       <c r="D204" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E204" s="11"/>
       <c r="F204" s="8"/>
@@ -7761,7 +7749,7 @@
         <v>2</v>
       </c>
       <c r="D205" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E205" s="11"/>
       <c r="F205" s="8"/>
@@ -7778,7 +7766,7 @@
         <v>1</v>
       </c>
       <c r="D206" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E206" s="11"/>
       <c r="F206" s="8"/>
@@ -7795,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="D207" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E207" s="11"/>
       <c r="F207" s="8"/>
@@ -7812,7 +7800,7 @@
         <v>1</v>
       </c>
       <c r="D208" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E208" s="11"/>
       <c r="F208" s="8"/>
@@ -7829,7 +7817,7 @@
         <v>1</v>
       </c>
       <c r="D209" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E209" s="11"/>
       <c r="F209" s="8"/>
@@ -7840,7 +7828,7 @@
         <v>42</v>
       </c>
       <c r="B210" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C210" s="8">
         <v>542</v>
@@ -7855,7 +7843,7 @@
         <v>42</v>
       </c>
       <c r="B211" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C211" s="8">
         <v>418</v>
@@ -7870,7 +7858,7 @@
         <v>42</v>
       </c>
       <c r="B212" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C212" s="8">
         <v>292</v>
@@ -7885,7 +7873,7 @@
         <v>42</v>
       </c>
       <c r="B213" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C213" s="8">
         <v>203</v>
@@ -7930,7 +7918,7 @@
         <v>42</v>
       </c>
       <c r="B216" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C216" s="8">
         <v>96</v>
@@ -7945,7 +7933,7 @@
         <v>42</v>
       </c>
       <c r="B217" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C217" s="8">
         <v>54</v>
@@ -7975,7 +7963,7 @@
         <v>42</v>
       </c>
       <c r="B219" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C219" s="8">
         <v>23</v>
@@ -8140,7 +8128,7 @@
         <v>39</v>
       </c>
       <c r="B230" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C230" s="8">
         <v>92</v>
@@ -8170,7 +8158,7 @@
         <v>39</v>
       </c>
       <c r="B232" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C232" s="8">
         <v>24</v>
@@ -8185,7 +8173,7 @@
         <v>39</v>
       </c>
       <c r="B233" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C233" s="8">
         <v>19</v>
@@ -8215,7 +8203,7 @@
         <v>39</v>
       </c>
       <c r="B235" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C235" s="8">
         <v>10</v>
@@ -8290,16 +8278,16 @@
         <v>41</v>
       </c>
       <c r="B240" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C240" s="8">
         <v>1183</v>
       </c>
       <c r="D240" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E240" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="F240" s="8"/>
       <c r="G240" s="8"/>
@@ -8315,7 +8303,7 @@
         <v>14</v>
       </c>
       <c r="D241" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E241" s="11"/>
       <c r="F241" s="8"/>
@@ -8326,13 +8314,13 @@
         <v>41</v>
       </c>
       <c r="B242" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C242" s="8">
         <v>13</v>
       </c>
       <c r="D242" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E242" s="11"/>
       <c r="F242" s="8"/>
@@ -8349,7 +8337,7 @@
         <v>13</v>
       </c>
       <c r="D243" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E243" s="11"/>
       <c r="F243" s="8"/>
@@ -8360,13 +8348,13 @@
         <v>41</v>
       </c>
       <c r="B244" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C244" s="8">
         <v>4</v>
       </c>
       <c r="D244" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E244" s="11"/>
       <c r="F244" s="8"/>
@@ -8383,7 +8371,7 @@
         <v>3</v>
       </c>
       <c r="D245" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E245" s="11"/>
       <c r="F245" s="8"/>
@@ -8394,16 +8382,16 @@
         <v>41</v>
       </c>
       <c r="B246" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C246" s="8">
         <v>1308</v>
       </c>
       <c r="D246" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E246" s="9" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F246" s="8"/>
       <c r="G246" s="8"/>
@@ -8419,7 +8407,7 @@
         <v>260</v>
       </c>
       <c r="D247" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E247" s="11"/>
       <c r="F247" s="8"/>
@@ -8430,13 +8418,13 @@
         <v>41</v>
       </c>
       <c r="B248" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C248" s="8">
         <v>179</v>
       </c>
       <c r="D248" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E248" s="11"/>
       <c r="F248" s="8"/>
@@ -8447,13 +8435,13 @@
         <v>41</v>
       </c>
       <c r="B249" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C249" s="8">
         <v>73</v>
       </c>
       <c r="D249" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E249" s="11"/>
       <c r="F249" s="8"/>
@@ -8470,7 +8458,7 @@
         <v>72</v>
       </c>
       <c r="D250" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E250" s="11"/>
       <c r="F250" s="8"/>
@@ -8481,13 +8469,13 @@
         <v>41</v>
       </c>
       <c r="B251" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C251" s="8">
         <v>57</v>
       </c>
       <c r="D251" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E251" s="11"/>
       <c r="F251" s="8"/>
@@ -8498,13 +8486,13 @@
         <v>41</v>
       </c>
       <c r="B252" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C252" s="8">
         <v>39</v>
       </c>
       <c r="D252" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E252" s="11"/>
       <c r="F252" s="8"/>
@@ -8515,13 +8503,13 @@
         <v>41</v>
       </c>
       <c r="B253" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C253" s="8">
         <v>37</v>
       </c>
       <c r="D253" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E253" s="11"/>
       <c r="F253" s="8"/>
@@ -8532,13 +8520,13 @@
         <v>41</v>
       </c>
       <c r="B254" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C254" s="8">
         <v>36</v>
       </c>
       <c r="D254" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E254" s="11"/>
       <c r="F254" s="8"/>
@@ -8549,13 +8537,13 @@
         <v>41</v>
       </c>
       <c r="B255" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C255" s="8">
         <v>14</v>
       </c>
       <c r="D255" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E255" s="11"/>
       <c r="F255" s="8"/>
@@ -8572,7 +8560,7 @@
         <v>13</v>
       </c>
       <c r="D256" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E256" s="11"/>
       <c r="F256" s="8"/>
@@ -8583,13 +8571,13 @@
         <v>41</v>
       </c>
       <c r="B257" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C257" s="8">
         <v>12</v>
       </c>
       <c r="D257" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E257" s="11"/>
       <c r="F257" s="8"/>
@@ -8600,13 +8588,13 @@
         <v>41</v>
       </c>
       <c r="B258" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C258" s="8">
         <v>11</v>
       </c>
       <c r="D258" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E258" s="11"/>
       <c r="F258" s="8"/>
@@ -8623,7 +8611,7 @@
         <v>9</v>
       </c>
       <c r="D259" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E259" s="11"/>
       <c r="F259" s="8"/>
@@ -8634,13 +8622,13 @@
         <v>41</v>
       </c>
       <c r="B260" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C260" s="8">
         <v>5</v>
       </c>
       <c r="D260" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E260" s="11"/>
       <c r="F260" s="8"/>
@@ -8651,13 +8639,13 @@
         <v>41</v>
       </c>
       <c r="B261" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C261" s="8">
         <v>3</v>
       </c>
       <c r="D261" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E261" s="11"/>
       <c r="F261" s="8"/>
@@ -8674,7 +8662,7 @@
         <v>2</v>
       </c>
       <c r="D262" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E262" s="11"/>
       <c r="F262" s="8"/>
@@ -8691,7 +8679,7 @@
         <v>2</v>
       </c>
       <c r="D263" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E263" s="11"/>
       <c r="F263" s="8"/>
@@ -8708,7 +8696,7 @@
         <v>1</v>
       </c>
       <c r="D264" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E264" s="11"/>
       <c r="F264" s="8"/>
@@ -8725,7 +8713,7 @@
         <v>1</v>
       </c>
       <c r="D265" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E265" s="11"/>
       <c r="F265" s="8"/>
@@ -8742,7 +8730,7 @@
         <v>1</v>
       </c>
       <c r="D266" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E266" s="11"/>
       <c r="F266" s="8"/>
@@ -8759,7 +8747,7 @@
         <v>1</v>
       </c>
       <c r="D267" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E267" s="11"/>
       <c r="F267" s="8"/>
@@ -8776,7 +8764,7 @@
         <v>1</v>
       </c>
       <c r="D268" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E268" s="11"/>
       <c r="F268" s="8"/>
@@ -8793,7 +8781,7 @@
         <v>1</v>
       </c>
       <c r="D269" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E269" s="11"/>
       <c r="F269" s="8"/>
@@ -8810,7 +8798,7 @@
         <v>1</v>
       </c>
       <c r="D270" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E270" s="11"/>
       <c r="F270" s="8"/>
@@ -8827,7 +8815,7 @@
         <v>1</v>
       </c>
       <c r="D271" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E271" s="11"/>
       <c r="F271" s="8"/>
@@ -8844,7 +8832,7 @@
         <v>1</v>
       </c>
       <c r="D272" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E272" s="11"/>
       <c r="F272" s="8"/>
@@ -8861,7 +8849,7 @@
         <v>1</v>
       </c>
       <c r="D273" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E273" s="11"/>
       <c r="F273" s="8"/>
@@ -8878,7 +8866,7 @@
         <v>1</v>
       </c>
       <c r="D274" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E274" s="11"/>
       <c r="F274" s="8"/>
@@ -8895,7 +8883,7 @@
         <v>1</v>
       </c>
       <c r="D275" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E275" s="11"/>
       <c r="F275" s="8"/>
@@ -8912,7 +8900,7 @@
         <v>1</v>
       </c>
       <c r="D276" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E276" s="11"/>
       <c r="F276" s="8"/>
@@ -8929,7 +8917,7 @@
         <v>1</v>
       </c>
       <c r="D277" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E277" s="11"/>
       <c r="F277" s="8"/>
@@ -8946,7 +8934,7 @@
         <v>1</v>
       </c>
       <c r="D278" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E278" s="11"/>
       <c r="F278" s="8"/>
@@ -8957,16 +8945,16 @@
         <v>41</v>
       </c>
       <c r="B279" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C279" s="8">
         <v>795</v>
       </c>
       <c r="D279" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E279" s="9" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F279" s="8"/>
       <c r="G279" s="8"/>
@@ -8976,13 +8964,13 @@
         <v>41</v>
       </c>
       <c r="B280" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C280" s="8">
         <v>205</v>
       </c>
       <c r="D280" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E280" s="11"/>
       <c r="F280" s="8"/>
@@ -8999,7 +8987,7 @@
         <v>117</v>
       </c>
       <c r="D281" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E281" s="11"/>
       <c r="F281" s="8"/>
@@ -9016,7 +9004,7 @@
         <v>90</v>
       </c>
       <c r="D282" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E282" s="11"/>
       <c r="F282" s="8"/>
@@ -9027,13 +9015,13 @@
         <v>41</v>
       </c>
       <c r="B283" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C283" s="8">
         <v>7</v>
       </c>
       <c r="D283" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E283" s="11"/>
       <c r="F283" s="8"/>
@@ -9050,7 +9038,7 @@
         <v>5</v>
       </c>
       <c r="D284" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E284" s="11"/>
       <c r="F284" s="8"/>
@@ -9061,13 +9049,13 @@
         <v>41</v>
       </c>
       <c r="B285" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C285" s="8">
         <v>3</v>
       </c>
       <c r="D285" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E285" s="11"/>
       <c r="F285" s="8"/>
@@ -9084,7 +9072,7 @@
         <v>1</v>
       </c>
       <c r="D286" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E286" s="11"/>
       <c r="F286" s="8"/>
@@ -9101,7 +9089,7 @@
         <v>1</v>
       </c>
       <c r="D287" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E287" s="11"/>
       <c r="F287" s="8"/>
@@ -9118,7 +9106,7 @@
         <v>1</v>
       </c>
       <c r="D288" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E288" s="11"/>
       <c r="F288" s="8"/>
@@ -9135,7 +9123,7 @@
         <v>1</v>
       </c>
       <c r="D289" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E289" s="11"/>
       <c r="F289" s="8"/>
@@ -9146,16 +9134,16 @@
         <v>41</v>
       </c>
       <c r="B290" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C290" s="8">
         <v>520</v>
       </c>
       <c r="D290" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="E290" s="9" t="s">
         <v>224</v>
-      </c>
-      <c r="E290" s="9" t="s">
-        <v>227</v>
       </c>
       <c r="F290" s="8"/>
       <c r="G290" s="8"/>
@@ -9165,13 +9153,13 @@
         <v>41</v>
       </c>
       <c r="B291" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C291" s="8">
         <v>455</v>
       </c>
       <c r="D291" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E291" s="11"/>
       <c r="F291" s="8"/>
@@ -9182,13 +9170,13 @@
         <v>41</v>
       </c>
       <c r="B292" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C292" s="8">
         <v>404</v>
       </c>
       <c r="D292" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E292" s="11"/>
       <c r="F292" s="8"/>
@@ -9199,13 +9187,13 @@
         <v>41</v>
       </c>
       <c r="B293" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C293" s="8">
         <v>94</v>
       </c>
       <c r="D293" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E293" s="11"/>
       <c r="F293" s="8"/>
@@ -9222,7 +9210,7 @@
         <v>32</v>
       </c>
       <c r="D294" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E294" s="11"/>
       <c r="F294" s="8"/>
@@ -9233,13 +9221,13 @@
         <v>41</v>
       </c>
       <c r="B295" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C295" s="8">
         <v>9</v>
       </c>
       <c r="D295" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E295" s="11"/>
       <c r="F295" s="8"/>
@@ -9256,7 +9244,7 @@
         <v>3</v>
       </c>
       <c r="D296" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E296" s="11"/>
       <c r="F296" s="8"/>
@@ -9273,7 +9261,7 @@
         <v>1</v>
       </c>
       <c r="D297" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E297" s="11"/>
       <c r="F297" s="8"/>
@@ -9290,7 +9278,7 @@
         <v>1</v>
       </c>
       <c r="D298" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E298" s="11"/>
       <c r="F298" s="8"/>
@@ -9307,7 +9295,7 @@
         <v>1</v>
       </c>
       <c r="D299" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E299" s="11"/>
       <c r="F299" s="8"/>
@@ -9324,7 +9312,7 @@
         <v>1</v>
       </c>
       <c r="D300" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E300" s="11"/>
       <c r="F300" s="8"/>
@@ -9336,7 +9324,7 @@
       <sortCondition ref="A1:A300"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="G2 F5:G5 F2:F300">
+  <conditionalFormatting sqref="G2 F2:F300 F5:G5">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Calibration of european seabass
</commit_message>
<xml_diff>
--- a/data/raw_data/feed_profiles_and_composition.xlsx
+++ b/data/raw_data/feed_profiles_and_composition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\climate_risks_to_fed_mariculture\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE24ADC3-867E-4C70-99C6-804B1D444301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EC04E6-4D6D-47D8-9A7E-C69B42F88450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24" yWindow="1236" windowWidth="20136" windowHeight="13908" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5268" yWindow="0" windowWidth="25236" windowHeight="16656" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="feed_formulations" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="228">
   <si>
     <t>ingredient</t>
   </si>
@@ -4558,7 +4558,7 @@
         <v>176</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G9" s="8"/>
     </row>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>177</v>
@@ -4599,7 +4599,9 @@
       <c r="E11" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="F11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -4616,7 +4618,9 @@
         <v>142</v>
       </c>
       <c r="E12" s="11"/>
-      <c r="F12" s="8"/>
+      <c r="F12" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -4633,7 +4637,9 @@
         <v>142</v>
       </c>
       <c r="E13" s="11"/>
-      <c r="F13" s="8"/>
+      <c r="F13" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -4650,7 +4656,9 @@
         <v>142</v>
       </c>
       <c r="E14" s="11"/>
-      <c r="F14" s="8"/>
+      <c r="F14" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G14" s="8"/>
     </row>
     <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -4667,7 +4675,9 @@
         <v>142</v>
       </c>
       <c r="E15" s="11"/>
-      <c r="F15" s="8"/>
+      <c r="F15" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:7" ht="26.4" hidden="1" x14ac:dyDescent="0.25">
@@ -7283,7 +7293,7 @@
       </c>
       <c r="G177" s="8"/>
     </row>
-    <row r="178" spans="1:7" ht="52.8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A178" s="8" t="s">
         <v>82</v>
       </c>
@@ -7304,7 +7314,7 @@
       </c>
       <c r="G178" s="8"/>
     </row>
-    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="8" t="s">
         <v>82</v>
       </c>
@@ -7323,7 +7333,7 @@
       </c>
       <c r="G179" s="8"/>
     </row>
-    <row r="180" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="8" t="s">
         <v>82</v>
       </c>
@@ -7342,7 +7352,7 @@
       </c>
       <c r="G180" s="8"/>
     </row>
-    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="8" t="s">
         <v>82</v>
       </c>
@@ -7361,7 +7371,7 @@
       </c>
       <c r="G181" s="8"/>
     </row>
-    <row r="182" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="8" t="s">
         <v>82</v>
       </c>
@@ -7380,7 +7390,7 @@
       </c>
       <c r="G182" s="8"/>
     </row>
-    <row r="183" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" s="8" t="s">
         <v>82</v>
       </c>
@@ -7399,7 +7409,7 @@
       </c>
       <c r="G183" s="8"/>
     </row>
-    <row r="184" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" s="8" t="s">
         <v>82</v>
       </c>
@@ -7418,7 +7428,7 @@
       </c>
       <c r="G184" s="8"/>
     </row>
-    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
         <v>82</v>
       </c>
@@ -7437,7 +7447,7 @@
       </c>
       <c r="G185" s="8"/>
     </row>
-    <row r="186" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="8" t="s">
         <v>82</v>
       </c>
@@ -7456,7 +7466,7 @@
       </c>
       <c r="G186" s="8"/>
     </row>
-    <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="8" t="s">
         <v>82</v>
       </c>
@@ -7475,7 +7485,7 @@
       </c>
       <c r="G187" s="8"/>
     </row>
-    <row r="188" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="8" t="s">
         <v>82</v>
       </c>
@@ -7494,7 +7504,7 @@
       </c>
       <c r="G188" s="8"/>
     </row>
-    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="8" t="s">
         <v>82</v>
       </c>
@@ -7513,7 +7523,7 @@
       </c>
       <c r="G189" s="8"/>
     </row>
-    <row r="190" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="8" t="s">
         <v>82</v>
       </c>
@@ -7532,7 +7542,7 @@
       </c>
       <c r="G190" s="8"/>
     </row>
-    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="8" t="s">
         <v>82</v>
       </c>
@@ -7551,7 +7561,7 @@
       </c>
       <c r="G191" s="8"/>
     </row>
-    <row r="192" spans="1:7" ht="52.8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A192" s="8" t="s">
         <v>82</v>
       </c>
@@ -7570,7 +7580,7 @@
       <c r="F192" s="8"/>
       <c r="G192" s="8"/>
     </row>
-    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" s="8" t="s">
         <v>82</v>
       </c>
@@ -7587,7 +7597,7 @@
       <c r="F193" s="8"/>
       <c r="G193" s="8"/>
     </row>
-    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="8" t="s">
         <v>82</v>
       </c>
@@ -7604,7 +7614,7 @@
       <c r="F194" s="8"/>
       <c r="G194" s="8"/>
     </row>
-    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="8" t="s">
         <v>82</v>
       </c>
@@ -7621,7 +7631,7 @@
       <c r="F195" s="8"/>
       <c r="G195" s="8"/>
     </row>
-    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="8" t="s">
         <v>82</v>
       </c>
@@ -7638,7 +7648,7 @@
       <c r="F196" s="8"/>
       <c r="G196" s="8"/>
     </row>
-    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="8" t="s">
         <v>82</v>
       </c>
@@ -7655,7 +7665,7 @@
       <c r="F197" s="8"/>
       <c r="G197" s="8"/>
     </row>
-    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" s="8" t="s">
         <v>82</v>
       </c>
@@ -7672,7 +7682,7 @@
       <c r="F198" s="8"/>
       <c r="G198" s="8"/>
     </row>
-    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" s="8" t="s">
         <v>82</v>
       </c>
@@ -7689,7 +7699,7 @@
       <c r="F199" s="8"/>
       <c r="G199" s="8"/>
     </row>
-    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" s="8" t="s">
         <v>82</v>
       </c>
@@ -7706,7 +7716,7 @@
       <c r="F200" s="8"/>
       <c r="G200" s="8"/>
     </row>
-    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" s="8" t="s">
         <v>82</v>
       </c>
@@ -7723,7 +7733,7 @@
       <c r="F201" s="8"/>
       <c r="G201" s="8"/>
     </row>
-    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" s="8" t="s">
         <v>82</v>
       </c>
@@ -7740,7 +7750,7 @@
       <c r="F202" s="8"/>
       <c r="G202" s="8"/>
     </row>
-    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" s="8" t="s">
         <v>82</v>
       </c>
@@ -7757,7 +7767,7 @@
       <c r="F203" s="8"/>
       <c r="G203" s="8"/>
     </row>
-    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" s="8" t="s">
         <v>82</v>
       </c>
@@ -7774,7 +7784,7 @@
       <c r="F204" s="8"/>
       <c r="G204" s="8"/>
     </row>
-    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="8" t="s">
         <v>82</v>
       </c>
@@ -7791,7 +7801,7 @@
       <c r="F205" s="8"/>
       <c r="G205" s="8"/>
     </row>
-    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="8" t="s">
         <v>82</v>
       </c>
@@ -7808,7 +7818,7 @@
       <c r="F206" s="8"/>
       <c r="G206" s="8"/>
     </row>
-    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="8" t="s">
         <v>82</v>
       </c>
@@ -7825,7 +7835,7 @@
       <c r="F207" s="8"/>
       <c r="G207" s="8"/>
     </row>
-    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="8" t="s">
         <v>82</v>
       </c>
@@ -7842,7 +7852,7 @@
       <c r="F208" s="8"/>
       <c r="G208" s="8"/>
     </row>
-    <row r="209" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" s="8" t="s">
         <v>82</v>
       </c>
@@ -8309,7 +8319,7 @@
       <c r="F239" s="8"/>
       <c r="G239" s="8"/>
     </row>
-    <row r="240" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="8" t="s">
         <v>41</v>
       </c>
@@ -8328,7 +8338,7 @@
       <c r="F240" s="8"/>
       <c r="G240" s="8"/>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="8" t="s">
         <v>41</v>
       </c>
@@ -8345,7 +8355,7 @@
       <c r="F241" s="8"/>
       <c r="G241" s="8"/>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="8" t="s">
         <v>41</v>
       </c>
@@ -8362,7 +8372,7 @@
       <c r="F242" s="8"/>
       <c r="G242" s="8"/>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="8" t="s">
         <v>41</v>
       </c>
@@ -8379,7 +8389,7 @@
       <c r="F243" s="8"/>
       <c r="G243" s="8"/>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="8" t="s">
         <v>41</v>
       </c>
@@ -8396,7 +8406,7 @@
       <c r="F244" s="8"/>
       <c r="G244" s="8"/>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" s="8" t="s">
         <v>41</v>
       </c>
@@ -8413,7 +8423,7 @@
       <c r="F245" s="8"/>
       <c r="G245" s="8"/>
     </row>
-    <row r="246" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" ht="52.8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="8" t="s">
         <v>41</v>
       </c>
@@ -8432,7 +8442,7 @@
       <c r="F246" s="8"/>
       <c r="G246" s="8"/>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="8" t="s">
         <v>41</v>
       </c>
@@ -8449,7 +8459,7 @@
       <c r="F247" s="8"/>
       <c r="G247" s="8"/>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" s="8" t="s">
         <v>41</v>
       </c>
@@ -8466,7 +8476,7 @@
       <c r="F248" s="8"/>
       <c r="G248" s="8"/>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="8" t="s">
         <v>41</v>
       </c>
@@ -8483,7 +8493,7 @@
       <c r="F249" s="8"/>
       <c r="G249" s="8"/>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" s="8" t="s">
         <v>41</v>
       </c>
@@ -8500,7 +8510,7 @@
       <c r="F250" s="8"/>
       <c r="G250" s="8"/>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" s="8" t="s">
         <v>41</v>
       </c>
@@ -8517,7 +8527,7 @@
       <c r="F251" s="8"/>
       <c r="G251" s="8"/>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="8" t="s">
         <v>41</v>
       </c>
@@ -8534,7 +8544,7 @@
       <c r="F252" s="8"/>
       <c r="G252" s="8"/>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="8" t="s">
         <v>41</v>
       </c>
@@ -8551,7 +8561,7 @@
       <c r="F253" s="8"/>
       <c r="G253" s="8"/>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" s="8" t="s">
         <v>41</v>
       </c>
@@ -8568,7 +8578,7 @@
       <c r="F254" s="8"/>
       <c r="G254" s="8"/>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" s="8" t="s">
         <v>41</v>
       </c>
@@ -8585,7 +8595,7 @@
       <c r="F255" s="8"/>
       <c r="G255" s="8"/>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" s="8" t="s">
         <v>41</v>
       </c>
@@ -8602,7 +8612,7 @@
       <c r="F256" s="8"/>
       <c r="G256" s="8"/>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" s="8" t="s">
         <v>41</v>
       </c>
@@ -8619,7 +8629,7 @@
       <c r="F257" s="8"/>
       <c r="G257" s="8"/>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" s="8" t="s">
         <v>41</v>
       </c>
@@ -8636,7 +8646,7 @@
       <c r="F258" s="8"/>
       <c r="G258" s="8"/>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" s="8" t="s">
         <v>41</v>
       </c>
@@ -8653,7 +8663,7 @@
       <c r="F259" s="8"/>
       <c r="G259" s="8"/>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" s="8" t="s">
         <v>41</v>
       </c>
@@ -8670,7 +8680,7 @@
       <c r="F260" s="8"/>
       <c r="G260" s="8"/>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="8" t="s">
         <v>41</v>
       </c>
@@ -8687,7 +8697,7 @@
       <c r="F261" s="8"/>
       <c r="G261" s="8"/>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" s="8" t="s">
         <v>41</v>
       </c>
@@ -8704,7 +8714,7 @@
       <c r="F262" s="8"/>
       <c r="G262" s="8"/>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" s="8" t="s">
         <v>41</v>
       </c>
@@ -8721,7 +8731,7 @@
       <c r="F263" s="8"/>
       <c r="G263" s="8"/>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="8" t="s">
         <v>41</v>
       </c>
@@ -8738,7 +8748,7 @@
       <c r="F264" s="8"/>
       <c r="G264" s="8"/>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="8" t="s">
         <v>41</v>
       </c>
@@ -8755,7 +8765,7 @@
       <c r="F265" s="8"/>
       <c r="G265" s="8"/>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" s="8" t="s">
         <v>41</v>
       </c>
@@ -8772,7 +8782,7 @@
       <c r="F266" s="8"/>
       <c r="G266" s="8"/>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="8" t="s">
         <v>41</v>
       </c>
@@ -8789,7 +8799,7 @@
       <c r="F267" s="8"/>
       <c r="G267" s="8"/>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" s="8" t="s">
         <v>41</v>
       </c>
@@ -8806,7 +8816,7 @@
       <c r="F268" s="8"/>
       <c r="G268" s="8"/>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="8" t="s">
         <v>41</v>
       </c>
@@ -8823,7 +8833,7 @@
       <c r="F269" s="8"/>
       <c r="G269" s="8"/>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" s="8" t="s">
         <v>41</v>
       </c>
@@ -8840,7 +8850,7 @@
       <c r="F270" s="8"/>
       <c r="G270" s="8"/>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" s="8" t="s">
         <v>41</v>
       </c>
@@ -8857,7 +8867,7 @@
       <c r="F271" s="8"/>
       <c r="G271" s="8"/>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" s="8" t="s">
         <v>41</v>
       </c>
@@ -8874,7 +8884,7 @@
       <c r="F272" s="8"/>
       <c r="G272" s="8"/>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" s="8" t="s">
         <v>41</v>
       </c>
@@ -8891,7 +8901,7 @@
       <c r="F273" s="8"/>
       <c r="G273" s="8"/>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" s="8" t="s">
         <v>41</v>
       </c>
@@ -8908,7 +8918,7 @@
       <c r="F274" s="8"/>
       <c r="G274" s="8"/>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" s="8" t="s">
         <v>41</v>
       </c>
@@ -8925,7 +8935,7 @@
       <c r="F275" s="8"/>
       <c r="G275" s="8"/>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" s="8" t="s">
         <v>41</v>
       </c>
@@ -8942,7 +8952,7 @@
       <c r="F276" s="8"/>
       <c r="G276" s="8"/>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" s="8" t="s">
         <v>41</v>
       </c>
@@ -8959,7 +8969,7 @@
       <c r="F277" s="8"/>
       <c r="G277" s="8"/>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" s="8" t="s">
         <v>41</v>
       </c>
@@ -8976,7 +8986,7 @@
       <c r="F278" s="8"/>
       <c r="G278" s="8"/>
     </row>
-    <row r="279" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" s="8" t="s">
         <v>41</v>
       </c>
@@ -8995,7 +9005,7 @@
       <c r="F279" s="8"/>
       <c r="G279" s="8"/>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" s="8" t="s">
         <v>41</v>
       </c>
@@ -9012,7 +9022,7 @@
       <c r="F280" s="8"/>
       <c r="G280" s="8"/>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="8" t="s">
         <v>41</v>
       </c>
@@ -9029,7 +9039,7 @@
       <c r="F281" s="8"/>
       <c r="G281" s="8"/>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="8" t="s">
         <v>41</v>
       </c>
@@ -9046,7 +9056,7 @@
       <c r="F282" s="8"/>
       <c r="G282" s="8"/>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" s="8" t="s">
         <v>41</v>
       </c>
@@ -9063,7 +9073,7 @@
       <c r="F283" s="8"/>
       <c r="G283" s="8"/>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="8" t="s">
         <v>41</v>
       </c>
@@ -9080,7 +9090,7 @@
       <c r="F284" s="8"/>
       <c r="G284" s="8"/>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" s="8" t="s">
         <v>41</v>
       </c>
@@ -9097,7 +9107,7 @@
       <c r="F285" s="8"/>
       <c r="G285" s="8"/>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" s="8" t="s">
         <v>41</v>
       </c>
@@ -9114,7 +9124,7 @@
       <c r="F286" s="8"/>
       <c r="G286" s="8"/>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" s="8" t="s">
         <v>41</v>
       </c>
@@ -9131,7 +9141,7 @@
       <c r="F287" s="8"/>
       <c r="G287" s="8"/>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" s="8" t="s">
         <v>41</v>
       </c>
@@ -9148,7 +9158,7 @@
       <c r="F288" s="8"/>
       <c r="G288" s="8"/>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" s="8" t="s">
         <v>41</v>
       </c>
@@ -9165,7 +9175,7 @@
       <c r="F289" s="8"/>
       <c r="G289" s="8"/>
     </row>
-    <row r="290" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" s="8" t="s">
         <v>41</v>
       </c>
@@ -9184,7 +9194,7 @@
       <c r="F290" s="8"/>
       <c r="G290" s="8"/>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" s="8" t="s">
         <v>41</v>
       </c>
@@ -9201,7 +9211,7 @@
       <c r="F291" s="8"/>
       <c r="G291" s="8"/>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" s="8" t="s">
         <v>41</v>
       </c>
@@ -9218,7 +9228,7 @@
       <c r="F292" s="8"/>
       <c r="G292" s="8"/>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" s="8" t="s">
         <v>41</v>
       </c>
@@ -9235,7 +9245,7 @@
       <c r="F293" s="8"/>
       <c r="G293" s="8"/>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" s="8" t="s">
         <v>41</v>
       </c>
@@ -9252,7 +9262,7 @@
       <c r="F294" s="8"/>
       <c r="G294" s="8"/>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" s="8" t="s">
         <v>41</v>
       </c>
@@ -9269,7 +9279,7 @@
       <c r="F295" s="8"/>
       <c r="G295" s="8"/>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" s="8" t="s">
         <v>41</v>
       </c>
@@ -9286,7 +9296,7 @@
       <c r="F296" s="8"/>
       <c r="G296" s="8"/>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" s="8" t="s">
         <v>41</v>
       </c>
@@ -9303,7 +9313,7 @@
       <c r="F297" s="8"/>
       <c r="G297" s="8"/>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" s="8" t="s">
         <v>41</v>
       </c>
@@ -9320,7 +9330,7 @@
       <c r="F298" s="8"/>
       <c r="G298" s="8"/>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" s="8" t="s">
         <v>41</v>
       </c>
@@ -9337,7 +9347,7 @@
       <c r="F299" s="8"/>
       <c r="G299" s="8"/>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="8" t="s">
         <v>41</v>
       </c>
@@ -9358,14 +9368,14 @@
   <autoFilter ref="A1:G300" xr:uid="{38A162FC-7907-44C7-A909-E8E1323EC5F6}">
     <filterColumn colId="0">
       <filters>
-        <filter val="whiteleg_shrimp"/>
+        <filter val="seabream"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G300">
-      <sortCondition ref="A1:A300"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:G20">
+      <sortCondition ref="D1:D300"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="G2 F2:F300 F5:G5">
+  <conditionalFormatting sqref="G2 F5:G5 F2:F300">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Calibration for whiteleg shrimp
</commit_message>
<xml_diff>
--- a/data/raw_data/feed_profiles_and_composition.xlsx
+++ b/data/raw_data/feed_profiles_and_composition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\climate_risks_to_fed_mariculture\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EC04E6-4D6D-47D8-9A7E-C69B42F88450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F04F7CDA-7E3F-4F49-8F48-F42CF2E3EB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5268" yWindow="0" windowWidth="25236" windowHeight="16656" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25260" yWindow="1836" windowWidth="15528" windowHeight="13656" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="feed_formulations" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="228">
   <si>
     <t>ingredient</t>
   </si>
@@ -1143,7 +1143,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:N1097"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>49</v>
       </c>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>49</v>
       </c>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>49</v>
       </c>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>49</v>
       </c>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>49</v>
       </c>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>49</v>
       </c>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>49</v>
       </c>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>49</v>
       </c>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:14" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>49</v>
       </c>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>49</v>
       </c>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>49</v>
       </c>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>49</v>
       </c>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>49</v>
       </c>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>44</v>
       </c>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>44</v>
       </c>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>44</v>
       </c>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>44</v>
       </c>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>44</v>
       </c>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>44</v>
       </c>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="D27" s="2"/>
     </row>
-    <row r="28" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>44</v>
       </c>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D28" s="2"/>
     </row>
-    <row r="29" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>44</v>
       </c>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="D29" s="2"/>
     </row>
-    <row r="30" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>44</v>
       </c>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="D30" s="2"/>
     </row>
-    <row r="31" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>44</v>
       </c>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="D31" s="2"/>
     </row>
-    <row r="32" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>44</v>
       </c>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D32" s="2"/>
     </row>
-    <row r="33" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>44</v>
       </c>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="D33" s="2"/>
     </row>
-    <row r="34" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>44</v>
       </c>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="D34" s="2"/>
     </row>
-    <row r="35" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>44</v>
       </c>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D35" s="2"/>
     </row>
-    <row r="36" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>43</v>
       </c>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D36" s="2"/>
     </row>
-    <row r="37" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>43</v>
       </c>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="D37" s="2"/>
     </row>
-    <row r="38" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>43</v>
       </c>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="D38" s="2"/>
     </row>
-    <row r="39" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>43</v>
       </c>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="D39" s="2"/>
     </row>
-    <row r="40" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>43</v>
       </c>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="D40" s="2"/>
     </row>
-    <row r="41" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>43</v>
       </c>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D41" s="2"/>
     </row>
-    <row r="42" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>43</v>
       </c>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="D42" s="2"/>
     </row>
-    <row r="43" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="D43" s="2"/>
     </row>
-    <row r="44" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D44" s="2"/>
     </row>
-    <row r="45" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>43</v>
       </c>
@@ -1722,7 +1722,7 @@
       </c>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>43</v>
       </c>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>43</v>
       </c>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="D48" s="2"/>
     </row>
-    <row r="49" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>43</v>
       </c>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="D49" s="2"/>
     </row>
-    <row r="50" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>43</v>
       </c>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="D50" s="2"/>
     </row>
-    <row r="51" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>43</v>
       </c>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="D51" s="2"/>
     </row>
-    <row r="52" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>43</v>
       </c>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="D52" s="2"/>
     </row>
-    <row r="53" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>48</v>
       </c>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="D53" s="2"/>
     </row>
-    <row r="54" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>48</v>
       </c>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="D54" s="2"/>
     </row>
-    <row r="55" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>48</v>
       </c>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D55" s="2"/>
     </row>
-    <row r="56" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>48</v>
       </c>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D56" s="2"/>
     </row>
-    <row r="57" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>48</v>
       </c>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D57" s="2"/>
     </row>
-    <row r="58" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>48</v>
       </c>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="D58" s="2"/>
     </row>
-    <row r="59" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>48</v>
       </c>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="D59" s="2"/>
     </row>
-    <row r="60" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>48</v>
       </c>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D60" s="2"/>
     </row>
-    <row r="61" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>48</v>
       </c>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="D61" s="2"/>
     </row>
-    <row r="62" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>48</v>
       </c>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D62" s="2"/>
     </row>
-    <row r="63" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>48</v>
       </c>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="D63" s="2"/>
     </row>
-    <row r="64" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>48</v>
       </c>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="D64" s="2"/>
     </row>
-    <row r="65" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>198</v>
       </c>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D65" s="2"/>
     </row>
-    <row r="66" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>198</v>
       </c>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="D66" s="2"/>
     </row>
-    <row r="67" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>198</v>
       </c>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="D67" s="3"/>
     </row>
-    <row r="68" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>198</v>
       </c>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D68" s="2"/>
     </row>
-    <row r="69" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>198</v>
       </c>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="D69" s="2"/>
     </row>
-    <row r="70" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>198</v>
       </c>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="D70" s="2"/>
     </row>
-    <row r="71" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>198</v>
       </c>
@@ -2022,7 +2022,7 @@
       </c>
       <c r="D71" s="2"/>
     </row>
-    <row r="72" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>198</v>
       </c>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D72" s="2"/>
     </row>
-    <row r="73" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>198</v>
       </c>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="D73" s="2"/>
     </row>
-    <row r="74" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>198</v>
       </c>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D74" s="2"/>
     </row>
-    <row r="75" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>198</v>
       </c>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="D75" s="2"/>
     </row>
-    <row r="76" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>198</v>
       </c>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="D76" s="2"/>
     </row>
-    <row r="77" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>210</v>
       </c>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="D77" s="3"/>
     </row>
-    <row r="78" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>210</v>
       </c>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="D78" s="3"/>
     </row>
-    <row r="79" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>210</v>
       </c>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D79" s="3"/>
     </row>
-    <row r="80" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>210</v>
       </c>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="D80" s="3"/>
     </row>
-    <row r="81" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>210</v>
       </c>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="D81" s="3"/>
     </row>
-    <row r="82" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>210</v>
       </c>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="D82" s="3"/>
     </row>
-    <row r="83" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>210</v>
       </c>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="D83" s="3"/>
     </row>
-    <row r="84" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>210</v>
       </c>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="D84" s="3"/>
     </row>
-    <row r="85" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>210</v>
       </c>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D85" s="3"/>
     </row>
-    <row r="86" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>210</v>
       </c>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="D86" s="3"/>
     </row>
-    <row r="87" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>210</v>
       </c>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="D87" s="3"/>
     </row>
-    <row r="88" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>30</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>33</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>33</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>33</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="92" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>33</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>33</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>33</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>29</v>
       </c>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="D95" s="2"/>
     </row>
-    <row r="96" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>203</v>
       </c>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="D96" s="3"/>
     </row>
-    <row r="97" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>203</v>
       </c>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="D97" s="3"/>
     </row>
-    <row r="98" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>203</v>
       </c>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="D98" s="3"/>
     </row>
-    <row r="99" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>203</v>
       </c>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="D99" s="3"/>
     </row>
-    <row r="100" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>203</v>
       </c>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="D100" s="3"/>
     </row>
-    <row r="101" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>203</v>
       </c>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="D101" s="3"/>
     </row>
-    <row r="102" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>203</v>
       </c>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D102" s="3"/>
     </row>
-    <row r="103" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>203</v>
       </c>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D103" s="3"/>
     </row>
-    <row r="104" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>203</v>
       </c>
@@ -2438,22 +2438,22 @@
       </c>
       <c r="D104" s="3"/>
     </row>
-    <row r="105" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="106" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="108" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>181</v>
       </c>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D108" s="3"/>
     </row>
-    <row r="109" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>181</v>
       </c>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="D109" s="3"/>
     </row>
-    <row r="110" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>181</v>
       </c>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="D110" s="3"/>
     </row>
-    <row r="111" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>181</v>
       </c>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="D111" s="3"/>
     </row>
-    <row r="112" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>181</v>
       </c>
@@ -2516,7 +2516,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="113" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>181</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="114" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>181</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="115" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>181</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>181</v>
       </c>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="D116" s="3"/>
     </row>
-    <row r="117" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>181</v>
       </c>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="D117" s="3"/>
     </row>
-    <row r="118" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>181</v>
       </c>
@@ -2597,7 +2597,7 @@
       </c>
       <c r="D118" s="3"/>
     </row>
-    <row r="119" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>181</v>
       </c>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="D119" s="3"/>
     </row>
-    <row r="120" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>181</v>
       </c>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="D120" s="3"/>
     </row>
-    <row r="121" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>181</v>
       </c>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="D121" s="3"/>
     </row>
-    <row r="122" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>179</v>
       </c>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="D122" s="3"/>
     </row>
-    <row r="123" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>179</v>
       </c>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="D123" s="3"/>
     </row>
-    <row r="124" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>179</v>
       </c>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="D124" s="3"/>
     </row>
-    <row r="125" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>179</v>
       </c>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="D125" s="3"/>
     </row>
-    <row r="126" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>179</v>
       </c>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="D126" s="3"/>
     </row>
-    <row r="127" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>179</v>
       </c>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="D127" s="3"/>
     </row>
-    <row r="128" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>179</v>
       </c>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="D128" s="3"/>
     </row>
-    <row r="129" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>179</v>
       </c>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="D129" s="3"/>
     </row>
-    <row r="130" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>179</v>
       </c>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D130" s="3"/>
     </row>
-    <row r="131" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>179</v>
       </c>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="D131" s="3"/>
     </row>
-    <row r="132" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>179</v>
       </c>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="D132" s="3"/>
     </row>
-    <row r="133" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>179</v>
       </c>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="D133" s="3"/>
     </row>
-    <row r="134" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>179</v>
       </c>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="D134" s="3"/>
     </row>
-    <row r="135" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>179</v>
       </c>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="D135" s="3"/>
     </row>
-    <row r="136" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>179</v>
       </c>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="D136" s="3"/>
     </row>
-    <row r="137" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>179</v>
       </c>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="D137" s="3"/>
     </row>
-    <row r="138" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>182</v>
       </c>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="D138" s="3"/>
     </row>
-    <row r="139" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>182</v>
       </c>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="D139" s="3"/>
     </row>
-    <row r="140" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>182</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>182</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>182</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>182</v>
       </c>
@@ -2909,7 +2909,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>182</v>
       </c>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="D144" s="3"/>
     </row>
-    <row r="145" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>182</v>
       </c>
@@ -2933,7 +2933,7 @@
       </c>
       <c r="D145" s="3"/>
     </row>
-    <row r="146" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>182</v>
       </c>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="D146" s="3"/>
     </row>
-    <row r="147" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>182</v>
       </c>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="D147" s="3"/>
     </row>
-    <row r="148" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>182</v>
       </c>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="D148" s="3"/>
     </row>
-    <row r="149" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>182</v>
       </c>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="D149" s="3"/>
     </row>
-    <row r="150" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>195</v>
       </c>
@@ -2993,7 +2993,7 @@
       </c>
       <c r="D150" s="2"/>
     </row>
-    <row r="151" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>195</v>
       </c>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="D151" s="2"/>
     </row>
-    <row r="152" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>195</v>
       </c>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="D152" s="2"/>
     </row>
-    <row r="153" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>195</v>
       </c>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="D153" s="2"/>
     </row>
-    <row r="154" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>195</v>
       </c>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D154" s="2"/>
     </row>
-    <row r="155" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>195</v>
       </c>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="D155" s="2"/>
     </row>
-    <row r="156" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>195</v>
       </c>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="D156" s="2"/>
     </row>
-    <row r="157" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>191</v>
       </c>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="D157" s="3"/>
     </row>
-    <row r="158" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>191</v>
       </c>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="D158" s="2"/>
     </row>
-    <row r="159" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>191</v>
       </c>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="D159" s="2"/>
     </row>
-    <row r="160" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>191</v>
       </c>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="D160" s="2"/>
     </row>
-    <row r="161" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>191</v>
       </c>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="D161" s="2"/>
     </row>
-    <row r="162" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>191</v>
       </c>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="D162" s="2"/>
     </row>
-    <row r="163" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>191</v>
       </c>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="D163" s="2"/>
     </row>
-    <row r="164" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>191</v>
       </c>
@@ -3162,17 +3162,17 @@
       </c>
       <c r="D164" s="2"/>
     </row>
-    <row r="165" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="166" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="167" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>211</v>
       </c>
@@ -3183,7 +3183,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="168" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>211</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="169" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>211</v>
       </c>
@@ -3205,7 +3205,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="170" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>211</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>2.9999999999999805E-2</v>
       </c>
     </row>
-    <row r="171" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>211</v>
       </c>
@@ -3227,7 +3227,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="172" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>211</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="173" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>211</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="174" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>214</v>
       </c>
@@ -3260,7 +3260,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="175" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>214</v>
       </c>
@@ -3271,7 +3271,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:4" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>214</v>
       </c>
@@ -3282,7 +3282,7 @@
         <v>5.5999999999998273E-3</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>214</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>0.17500000000000002</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>214</v>
       </c>
@@ -3304,7 +3304,7 @@
         <v>0.45140000000000002</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>216</v>
       </c>
@@ -3315,7 +3315,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>216</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>216</v>
       </c>
@@ -3337,7 +3337,7 @@
         <v>0.1474</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>216</v>
       </c>
@@ -3348,7 +3348,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>216</v>
       </c>
@@ -3359,7 +3359,7 @@
         <v>3.1000000000000028E-2</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>216</v>
       </c>
@@ -3370,7 +3370,7 @@
         <v>1.15E-2</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>216</v>
       </c>
@@ -3381,7 +3381,7 @@
         <v>0.47010000000000002</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>222</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>222</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>222</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>9.2999999999999972E-2</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>222</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>0.20300000000000001</v>
       </c>
     </row>
-    <row r="190" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>222</v>
       </c>
@@ -3437,7 +3437,7 @@
         <v>0.21500000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>222</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" ht="13.2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>222</v>
       </c>
@@ -4366,6 +4366,11 @@
     <row r="1097" ht="13.2" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:D192" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="asian_seabass-china"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A167:D192">
       <sortCondition ref="A1:A192"/>
     </sortState>
@@ -4381,12 +4386,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38A162FC-7907-44C7-A909-E8E1323EC5F6}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G300"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.21875" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.5546875" style="7" customWidth="1"/>
     <col min="3" max="3" width="11.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.88671875" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="100.77734375" style="10" customWidth="1"/>
@@ -4418,7 +4422,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>199</v>
       </c>
@@ -4437,7 +4441,7 @@
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>199</v>
       </c>
@@ -4454,7 +4458,7 @@
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>199</v>
       </c>
@@ -4471,7 +4475,7 @@
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>199</v>
       </c>
@@ -4488,7 +4492,7 @@
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
     </row>
-    <row r="6" spans="1:7" ht="26.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>128</v>
       </c>
@@ -4507,7 +4511,7 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>128</v>
       </c>
@@ -4524,7 +4528,7 @@
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>128</v>
       </c>
@@ -4541,7 +4545,7 @@
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
     </row>
-    <row r="9" spans="1:7" ht="26.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>128</v>
       </c>
@@ -4562,7 +4566,7 @@
       </c>
       <c r="G9" s="8"/>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>128</v>
       </c>
@@ -4583,7 +4587,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="26.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>128</v>
       </c>
@@ -4604,7 +4608,7 @@
       </c>
       <c r="G11" s="8"/>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>128</v>
       </c>
@@ -4623,7 +4627,7 @@
       </c>
       <c r="G12" s="8"/>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>128</v>
       </c>
@@ -4642,7 +4646,7 @@
       </c>
       <c r="G13" s="8"/>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>128</v>
       </c>
@@ -4661,7 +4665,7 @@
       </c>
       <c r="G14" s="8"/>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>128</v>
       </c>
@@ -4680,7 +4684,7 @@
       </c>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:7" ht="26.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>128</v>
       </c>
@@ -4699,7 +4703,7 @@
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>128</v>
       </c>
@@ -4716,7 +4720,7 @@
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>128</v>
       </c>
@@ -4733,7 +4737,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>128</v>
       </c>
@@ -4750,7 +4754,7 @@
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>128</v>
       </c>
@@ -4767,7 +4771,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>119</v>
       </c>
@@ -4782,7 +4786,7 @@
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>119</v>
       </c>
@@ -4797,7 +4801,7 @@
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>119</v>
       </c>
@@ -4812,7 +4816,7 @@
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>119</v>
       </c>
@@ -4827,7 +4831,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>119</v>
       </c>
@@ -4842,7 +4846,7 @@
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
     </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>119</v>
       </c>
@@ -4857,7 +4861,7 @@
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
     </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>119</v>
       </c>
@@ -4872,7 +4876,7 @@
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
     </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>119</v>
       </c>
@@ -4887,7 +4891,7 @@
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
     </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>119</v>
       </c>
@@ -4902,7 +4906,7 @@
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>119</v>
       </c>
@@ -4917,7 +4921,7 @@
       <c r="F30" s="8"/>
       <c r="G30" s="8"/>
     </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>119</v>
       </c>
@@ -4932,7 +4936,7 @@
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
     </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>119</v>
       </c>
@@ -4947,7 +4951,7 @@
       <c r="F32" s="8"/>
       <c r="G32" s="8"/>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>119</v>
       </c>
@@ -4962,7 +4966,7 @@
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
     </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>119</v>
       </c>
@@ -4977,7 +4981,7 @@
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>119</v>
       </c>
@@ -4992,7 +4996,7 @@
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>119</v>
       </c>
@@ -5007,7 +5011,7 @@
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>119</v>
       </c>
@@ -5022,7 +5026,7 @@
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>119</v>
       </c>
@@ -5037,7 +5041,7 @@
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
     </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>119</v>
       </c>
@@ -5052,7 +5056,7 @@
       <c r="F39" s="8"/>
       <c r="G39" s="8"/>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>119</v>
       </c>
@@ -5067,7 +5071,7 @@
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>119</v>
       </c>
@@ -5082,7 +5086,7 @@
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>119</v>
       </c>
@@ -5097,7 +5101,7 @@
       <c r="F42" s="8"/>
       <c r="G42" s="8"/>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
         <v>119</v>
       </c>
@@ -5112,7 +5116,7 @@
       <c r="F43" s="8"/>
       <c r="G43" s="8"/>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
         <v>119</v>
       </c>
@@ -5127,7 +5131,7 @@
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
         <v>119</v>
       </c>
@@ -5142,7 +5146,7 @@
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
         <v>119</v>
       </c>
@@ -5157,7 +5161,7 @@
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
     </row>
-    <row r="47" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
         <v>118</v>
       </c>
@@ -5176,7 +5180,7 @@
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>118</v>
       </c>
@@ -5193,7 +5197,7 @@
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
     </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>118</v>
       </c>
@@ -5210,7 +5214,7 @@
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
     </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>118</v>
       </c>
@@ -5227,7 +5231,7 @@
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
     </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
         <v>118</v>
       </c>
@@ -5244,7 +5248,7 @@
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
     </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
         <v>118</v>
       </c>
@@ -5261,7 +5265,7 @@
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
     </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
         <v>118</v>
       </c>
@@ -5278,7 +5282,7 @@
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
     </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
         <v>118</v>
       </c>
@@ -5295,7 +5299,7 @@
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
     </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>118</v>
       </c>
@@ -5312,7 +5316,7 @@
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
     </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>118</v>
       </c>
@@ -5329,7 +5333,7 @@
       <c r="F56" s="8"/>
       <c r="G56" s="8"/>
     </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>118</v>
       </c>
@@ -5346,7 +5350,7 @@
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
     </row>
-    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>118</v>
       </c>
@@ -5363,7 +5367,7 @@
       <c r="F58" s="8"/>
       <c r="G58" s="8"/>
     </row>
-    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
         <v>118</v>
       </c>
@@ -5380,7 +5384,7 @@
       <c r="F59" s="8"/>
       <c r="G59" s="8"/>
     </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
         <v>118</v>
       </c>
@@ -5397,7 +5401,7 @@
       <c r="F60" s="8"/>
       <c r="G60" s="8"/>
     </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
         <v>118</v>
       </c>
@@ -5414,7 +5418,7 @@
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
     </row>
-    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
         <v>118</v>
       </c>
@@ -5431,7 +5435,7 @@
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
     </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
         <v>118</v>
       </c>
@@ -5448,7 +5452,7 @@
       <c r="F63" s="8"/>
       <c r="G63" s="8"/>
     </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
         <v>118</v>
       </c>
@@ -5465,7 +5469,7 @@
       <c r="F64" s="8"/>
       <c r="G64" s="8"/>
     </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
         <v>118</v>
       </c>
@@ -5482,7 +5486,7 @@
       <c r="F65" s="8"/>
       <c r="G65" s="8"/>
     </row>
-    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
         <v>118</v>
       </c>
@@ -5499,7 +5503,7 @@
       <c r="F66" s="8"/>
       <c r="G66" s="8"/>
     </row>
-    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
         <v>118</v>
       </c>
@@ -5516,7 +5520,7 @@
       <c r="F67" s="8"/>
       <c r="G67" s="8"/>
     </row>
-    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
         <v>118</v>
       </c>
@@ -5533,7 +5537,7 @@
       <c r="F68" s="8"/>
       <c r="G68" s="8"/>
     </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
         <v>118</v>
       </c>
@@ -5550,7 +5554,7 @@
       <c r="F69" s="8"/>
       <c r="G69" s="8"/>
     </row>
-    <row r="70" spans="1:7" ht="52.8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
         <v>117</v>
       </c>
@@ -5569,7 +5573,7 @@
       <c r="F70" s="8"/>
       <c r="G70" s="8"/>
     </row>
-    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
         <v>117</v>
       </c>
@@ -5586,7 +5590,7 @@
       <c r="F71" s="8"/>
       <c r="G71" s="8"/>
     </row>
-    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
         <v>117</v>
       </c>
@@ -5603,7 +5607,7 @@
       <c r="F72" s="8"/>
       <c r="G72" s="8"/>
     </row>
-    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
         <v>117</v>
       </c>
@@ -5620,7 +5624,7 @@
       <c r="F73" s="8"/>
       <c r="G73" s="8"/>
     </row>
-    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
         <v>117</v>
       </c>
@@ -5637,7 +5641,7 @@
       <c r="F74" s="8"/>
       <c r="G74" s="8"/>
     </row>
-    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
         <v>117</v>
       </c>
@@ -5654,7 +5658,7 @@
       <c r="F75" s="8"/>
       <c r="G75" s="8"/>
     </row>
-    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="8" t="s">
         <v>117</v>
       </c>
@@ -5671,7 +5675,7 @@
       <c r="F76" s="8"/>
       <c r="G76" s="8"/>
     </row>
-    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
         <v>117</v>
       </c>
@@ -5688,7 +5692,7 @@
       <c r="F77" s="8"/>
       <c r="G77" s="8"/>
     </row>
-    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
         <v>113</v>
       </c>
@@ -5703,7 +5707,7 @@
       <c r="F78" s="8"/>
       <c r="G78" s="8"/>
     </row>
-    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
         <v>113</v>
       </c>
@@ -5718,7 +5722,7 @@
       <c r="F79" s="8"/>
       <c r="G79" s="8"/>
     </row>
-    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="8" t="s">
         <v>113</v>
       </c>
@@ -5733,7 +5737,7 @@
       <c r="F80" s="8"/>
       <c r="G80" s="8"/>
     </row>
-    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
         <v>113</v>
       </c>
@@ -5748,7 +5752,7 @@
       <c r="F81" s="8"/>
       <c r="G81" s="8"/>
     </row>
-    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
         <v>113</v>
       </c>
@@ -5763,7 +5767,7 @@
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
     </row>
-    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
         <v>113</v>
       </c>
@@ -5778,7 +5782,7 @@
       <c r="F83" s="8"/>
       <c r="G83" s="8"/>
     </row>
-    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="8" t="s">
         <v>113</v>
       </c>
@@ -5793,7 +5797,7 @@
       <c r="F84" s="8"/>
       <c r="G84" s="8"/>
     </row>
-    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
         <v>113</v>
       </c>
@@ -5808,7 +5812,7 @@
       <c r="F85" s="8"/>
       <c r="G85" s="8"/>
     </row>
-    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="8" t="s">
         <v>113</v>
       </c>
@@ -5823,7 +5827,7 @@
       <c r="F86" s="8"/>
       <c r="G86" s="8"/>
     </row>
-    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
         <v>113</v>
       </c>
@@ -5838,7 +5842,7 @@
       <c r="F87" s="8"/>
       <c r="G87" s="8"/>
     </row>
-    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="8" t="s">
         <v>113</v>
       </c>
@@ -5853,7 +5857,7 @@
       <c r="F88" s="8"/>
       <c r="G88" s="8"/>
     </row>
-    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
         <v>113</v>
       </c>
@@ -5868,7 +5872,7 @@
       <c r="F89" s="8"/>
       <c r="G89" s="8"/>
     </row>
-    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
         <v>113</v>
       </c>
@@ -5883,7 +5887,7 @@
       <c r="F90" s="8"/>
       <c r="G90" s="8"/>
     </row>
-    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
         <v>113</v>
       </c>
@@ -5898,7 +5902,7 @@
       <c r="F91" s="8"/>
       <c r="G91" s="8"/>
     </row>
-    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="8" t="s">
         <v>113</v>
       </c>
@@ -5913,7 +5917,7 @@
       <c r="F92" s="8"/>
       <c r="G92" s="8"/>
     </row>
-    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
         <v>113</v>
       </c>
@@ -5928,7 +5932,7 @@
       <c r="F93" s="8"/>
       <c r="G93" s="8"/>
     </row>
-    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
         <v>33</v>
       </c>
@@ -5943,7 +5947,7 @@
       <c r="F94" s="8"/>
       <c r="G94" s="8"/>
     </row>
-    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
         <v>33</v>
       </c>
@@ -5958,7 +5962,7 @@
       <c r="F95" s="8"/>
       <c r="G95" s="8"/>
     </row>
-    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="8" t="s">
         <v>33</v>
       </c>
@@ -5973,7 +5977,7 @@
       <c r="F96" s="8"/>
       <c r="G96" s="8"/>
     </row>
-    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
         <v>33</v>
       </c>
@@ -5988,7 +5992,7 @@
       <c r="F97" s="8"/>
       <c r="G97" s="8"/>
     </row>
-    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="8" t="s">
         <v>33</v>
       </c>
@@ -6003,7 +6007,7 @@
       <c r="F98" s="8"/>
       <c r="G98" s="8"/>
     </row>
-    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
         <v>33</v>
       </c>
@@ -6018,7 +6022,7 @@
       <c r="F99" s="8"/>
       <c r="G99" s="8"/>
     </row>
-    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="8" t="s">
         <v>33</v>
       </c>
@@ -6033,7 +6037,7 @@
       <c r="F100" s="8"/>
       <c r="G100" s="8"/>
     </row>
-    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
         <v>33</v>
       </c>
@@ -6048,7 +6052,7 @@
       <c r="F101" s="8"/>
       <c r="G101" s="8"/>
     </row>
-    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="8" t="s">
         <v>33</v>
       </c>
@@ -6063,7 +6067,7 @@
       <c r="F102" s="8"/>
       <c r="G102" s="8"/>
     </row>
-    <row r="103" spans="1:7" ht="66" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" ht="66" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
         <v>36</v>
       </c>
@@ -6082,7 +6086,7 @@
       <c r="F103" s="8"/>
       <c r="G103" s="8"/>
     </row>
-    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
         <v>36</v>
       </c>
@@ -6099,7 +6103,7 @@
       <c r="F104" s="8"/>
       <c r="G104" s="8"/>
     </row>
-    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
         <v>36</v>
       </c>
@@ -6116,7 +6120,7 @@
       <c r="F105" s="8"/>
       <c r="G105" s="8"/>
     </row>
-    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="8" t="s">
         <v>36</v>
       </c>
@@ -6133,7 +6137,7 @@
       <c r="F106" s="8"/>
       <c r="G106" s="8"/>
     </row>
-    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
         <v>36</v>
       </c>
@@ -6150,7 +6154,7 @@
       <c r="F107" s="8"/>
       <c r="G107" s="8"/>
     </row>
-    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
         <v>36</v>
       </c>
@@ -6167,7 +6171,7 @@
       <c r="F108" s="8"/>
       <c r="G108" s="8"/>
     </row>
-    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
         <v>36</v>
       </c>
@@ -6184,7 +6188,7 @@
       <c r="F109" s="8"/>
       <c r="G109" s="8"/>
     </row>
-    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="8" t="s">
         <v>36</v>
       </c>
@@ -6201,7 +6205,7 @@
       <c r="F110" s="8"/>
       <c r="G110" s="8"/>
     </row>
-    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
         <v>36</v>
       </c>
@@ -6218,7 +6222,7 @@
       <c r="F111" s="8"/>
       <c r="G111" s="8"/>
     </row>
-    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
         <v>36</v>
       </c>
@@ -6235,7 +6239,7 @@
       <c r="F112" s="8"/>
       <c r="G112" s="8"/>
     </row>
-    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
         <v>36</v>
       </c>
@@ -6252,7 +6256,7 @@
       <c r="F113" s="8"/>
       <c r="G113" s="8"/>
     </row>
-    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="8" t="s">
         <v>36</v>
       </c>
@@ -6269,7 +6273,7 @@
       <c r="F114" s="8"/>
       <c r="G114" s="8"/>
     </row>
-    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
         <v>36</v>
       </c>
@@ -6286,7 +6290,7 @@
       <c r="F115" s="8"/>
       <c r="G115" s="8"/>
     </row>
-    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="8" t="s">
         <v>36</v>
       </c>
@@ -6303,7 +6307,7 @@
       <c r="F116" s="8"/>
       <c r="G116" s="8"/>
     </row>
-    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
         <v>36</v>
       </c>
@@ -6320,7 +6324,7 @@
       <c r="F117" s="8"/>
       <c r="G117" s="8"/>
     </row>
-    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
         <v>36</v>
       </c>
@@ -6337,7 +6341,7 @@
       <c r="F118" s="8"/>
       <c r="G118" s="8"/>
     </row>
-    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
         <v>36</v>
       </c>
@@ -6354,7 +6358,7 @@
       <c r="F119" s="8"/>
       <c r="G119" s="8"/>
     </row>
-    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="8" t="s">
         <v>40</v>
       </c>
@@ -6369,7 +6373,7 @@
       <c r="F120" s="8"/>
       <c r="G120" s="8"/>
     </row>
-    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
         <v>40</v>
       </c>
@@ -6384,7 +6388,7 @@
       <c r="F121" s="8"/>
       <c r="G121" s="8"/>
     </row>
-    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="8" t="s">
         <v>40</v>
       </c>
@@ -6399,7 +6403,7 @@
       <c r="F122" s="8"/>
       <c r="G122" s="8"/>
     </row>
-    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="8" t="s">
         <v>40</v>
       </c>
@@ -6414,7 +6418,7 @@
       <c r="F123" s="8"/>
       <c r="G123" s="8"/>
     </row>
-    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="8" t="s">
         <v>40</v>
       </c>
@@ -6429,7 +6433,7 @@
       <c r="F124" s="8"/>
       <c r="G124" s="8"/>
     </row>
-    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
         <v>40</v>
       </c>
@@ -6444,7 +6448,7 @@
       <c r="F125" s="8"/>
       <c r="G125" s="8"/>
     </row>
-    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="8" t="s">
         <v>40</v>
       </c>
@@ -6459,7 +6463,7 @@
       <c r="F126" s="8"/>
       <c r="G126" s="8"/>
     </row>
-    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
         <v>40</v>
       </c>
@@ -6474,7 +6478,7 @@
       <c r="F127" s="8"/>
       <c r="G127" s="8"/>
     </row>
-    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="8" t="s">
         <v>40</v>
       </c>
@@ -6489,7 +6493,7 @@
       <c r="F128" s="8"/>
       <c r="G128" s="8"/>
     </row>
-    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
         <v>40</v>
       </c>
@@ -6504,7 +6508,7 @@
       <c r="F129" s="8"/>
       <c r="G129" s="8"/>
     </row>
-    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="8" t="s">
         <v>40</v>
       </c>
@@ -6519,7 +6523,7 @@
       <c r="F130" s="8"/>
       <c r="G130" s="8"/>
     </row>
-    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="8" t="s">
         <v>40</v>
       </c>
@@ -6534,7 +6538,7 @@
       <c r="F131" s="8"/>
       <c r="G131" s="8"/>
     </row>
-    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="8" t="s">
         <v>40</v>
       </c>
@@ -6549,7 +6553,7 @@
       <c r="F132" s="8"/>
       <c r="G132" s="8"/>
     </row>
-    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="8" t="s">
         <v>40</v>
       </c>
@@ -6564,7 +6568,7 @@
       <c r="F133" s="8"/>
       <c r="G133" s="8"/>
     </row>
-    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="8" t="s">
         <v>40</v>
       </c>
@@ -6579,7 +6583,7 @@
       <c r="F134" s="8"/>
       <c r="G134" s="8"/>
     </row>
-    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="8" t="s">
         <v>40</v>
       </c>
@@ -6594,7 +6598,7 @@
       <c r="F135" s="8"/>
       <c r="G135" s="8"/>
     </row>
-    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="8" t="s">
         <v>40</v>
       </c>
@@ -6609,7 +6613,7 @@
       <c r="F136" s="8"/>
       <c r="G136" s="8"/>
     </row>
-    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
         <v>40</v>
       </c>
@@ -6624,7 +6628,7 @@
       <c r="F137" s="8"/>
       <c r="G137" s="8"/>
     </row>
-    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="8" t="s">
         <v>40</v>
       </c>
@@ -6639,7 +6643,7 @@
       <c r="F138" s="8"/>
       <c r="G138" s="8"/>
     </row>
-    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
         <v>40</v>
       </c>
@@ -6654,7 +6658,7 @@
       <c r="F139" s="8"/>
       <c r="G139" s="8"/>
     </row>
-    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="8" t="s">
         <v>40</v>
       </c>
@@ -6669,7 +6673,7 @@
       <c r="F140" s="8"/>
       <c r="G140" s="8"/>
     </row>
-    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="8" t="s">
         <v>40</v>
       </c>
@@ -6684,7 +6688,7 @@
       <c r="F141" s="8"/>
       <c r="G141" s="8"/>
     </row>
-    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="8" t="s">
         <v>40</v>
       </c>
@@ -6699,7 +6703,7 @@
       <c r="F142" s="8"/>
       <c r="G142" s="8"/>
     </row>
-    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="8" t="s">
         <v>37</v>
       </c>
@@ -6714,7 +6718,7 @@
       <c r="F143" s="8"/>
       <c r="G143" s="8"/>
     </row>
-    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="8" t="s">
         <v>37</v>
       </c>
@@ -6729,7 +6733,7 @@
       <c r="F144" s="8"/>
       <c r="G144" s="8"/>
     </row>
-    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="8" t="s">
         <v>37</v>
       </c>
@@ -6744,7 +6748,7 @@
       <c r="F145" s="8"/>
       <c r="G145" s="8"/>
     </row>
-    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="8" t="s">
         <v>37</v>
       </c>
@@ -6759,7 +6763,7 @@
       <c r="F146" s="8"/>
       <c r="G146" s="8"/>
     </row>
-    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="8" t="s">
         <v>37</v>
       </c>
@@ -6774,7 +6778,7 @@
       <c r="F147" s="8"/>
       <c r="G147" s="8"/>
     </row>
-    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="8" t="s">
         <v>37</v>
       </c>
@@ -6789,7 +6793,7 @@
       <c r="F148" s="8"/>
       <c r="G148" s="8"/>
     </row>
-    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="8" t="s">
         <v>37</v>
       </c>
@@ -6804,7 +6808,7 @@
       <c r="F149" s="8"/>
       <c r="G149" s="8"/>
     </row>
-    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="8" t="s">
         <v>37</v>
       </c>
@@ -6819,7 +6823,7 @@
       <c r="F150" s="8"/>
       <c r="G150" s="8"/>
     </row>
-    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
         <v>37</v>
       </c>
@@ -6834,7 +6838,7 @@
       <c r="F151" s="8"/>
       <c r="G151" s="8"/>
     </row>
-    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="8" t="s">
         <v>37</v>
       </c>
@@ -6849,7 +6853,7 @@
       <c r="F152" s="8"/>
       <c r="G152" s="8"/>
     </row>
-    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="8" t="s">
         <v>37</v>
       </c>
@@ -6864,7 +6868,7 @@
       <c r="F153" s="8"/>
       <c r="G153" s="8"/>
     </row>
-    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="8" t="s">
         <v>37</v>
       </c>
@@ -6879,7 +6883,7 @@
       <c r="F154" s="8"/>
       <c r="G154" s="8"/>
     </row>
-    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="8" t="s">
         <v>37</v>
       </c>
@@ -6894,7 +6898,7 @@
       <c r="F155" s="8"/>
       <c r="G155" s="8"/>
     </row>
-    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="8" t="s">
         <v>37</v>
       </c>
@@ -6909,7 +6913,7 @@
       <c r="F156" s="8"/>
       <c r="G156" s="8"/>
     </row>
-    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="8" t="s">
         <v>37</v>
       </c>
@@ -6924,7 +6928,7 @@
       <c r="F157" s="8"/>
       <c r="G157" s="8"/>
     </row>
-    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="8" t="s">
         <v>38</v>
       </c>
@@ -6939,7 +6943,7 @@
       <c r="F158" s="8"/>
       <c r="G158" s="8"/>
     </row>
-    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="8" t="s">
         <v>38</v>
       </c>
@@ -6954,7 +6958,7 @@
       <c r="F159" s="8"/>
       <c r="G159" s="8"/>
     </row>
-    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="8" t="s">
         <v>38</v>
       </c>
@@ -6969,7 +6973,7 @@
       <c r="F160" s="8"/>
       <c r="G160" s="8"/>
     </row>
-    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="8" t="s">
         <v>38</v>
       </c>
@@ -6984,7 +6988,7 @@
       <c r="F161" s="8"/>
       <c r="G161" s="8"/>
     </row>
-    <row r="162" spans="1:7" ht="26.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A162" s="8" t="s">
         <v>93</v>
       </c>
@@ -7005,7 +7009,7 @@
       </c>
       <c r="G162" s="8"/>
     </row>
-    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="8" t="s">
         <v>93</v>
       </c>
@@ -7023,7 +7027,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="8" t="s">
         <v>93</v>
       </c>
@@ -7042,7 +7046,7 @@
       </c>
       <c r="G164" s="8"/>
     </row>
-    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="8" t="s">
         <v>93</v>
       </c>
@@ -7061,7 +7065,7 @@
       </c>
       <c r="G165" s="8"/>
     </row>
-    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="8" t="s">
         <v>93</v>
       </c>
@@ -7080,7 +7084,7 @@
       </c>
       <c r="G166" s="8"/>
     </row>
-    <row r="167" spans="1:7" ht="52.8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A167" s="8" t="s">
         <v>93</v>
       </c>
@@ -7101,7 +7105,7 @@
       </c>
       <c r="G167" s="8"/>
     </row>
-    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="8" t="s">
         <v>93</v>
       </c>
@@ -7120,7 +7124,7 @@
       </c>
       <c r="G168" s="8"/>
     </row>
-    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="8" t="s">
         <v>93</v>
       </c>
@@ -7139,7 +7143,7 @@
       </c>
       <c r="G169" s="8"/>
     </row>
-    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="8" t="s">
         <v>93</v>
       </c>
@@ -7158,7 +7162,7 @@
       </c>
       <c r="G170" s="8"/>
     </row>
-    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="8" t="s">
         <v>93</v>
       </c>
@@ -7177,7 +7181,7 @@
       </c>
       <c r="G171" s="8"/>
     </row>
-    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="8" t="s">
         <v>93</v>
       </c>
@@ -7196,7 +7200,7 @@
       </c>
       <c r="G172" s="8"/>
     </row>
-    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
         <v>93</v>
       </c>
@@ -7215,7 +7219,7 @@
       </c>
       <c r="G173" s="8"/>
     </row>
-    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
         <v>93</v>
       </c>
@@ -7234,7 +7238,7 @@
       </c>
       <c r="G174" s="8"/>
     </row>
-    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
         <v>93</v>
       </c>
@@ -7253,7 +7257,7 @@
       </c>
       <c r="G175" s="8"/>
     </row>
-    <row r="176" spans="1:7" ht="52.8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
         <v>93</v>
       </c>
@@ -7274,7 +7278,7 @@
       </c>
       <c r="G176" s="8"/>
     </row>
-    <row r="177" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="8" t="s">
         <v>93</v>
       </c>
@@ -7310,7 +7314,7 @@
         <v>194</v>
       </c>
       <c r="F178" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G178" s="8"/>
     </row>
@@ -7329,7 +7333,7 @@
       </c>
       <c r="E179" s="11"/>
       <c r="F179" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G179" s="8"/>
     </row>
@@ -7348,7 +7352,7 @@
       </c>
       <c r="E180" s="11"/>
       <c r="F180" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G180" s="8"/>
     </row>
@@ -7367,7 +7371,7 @@
       </c>
       <c r="E181" s="11"/>
       <c r="F181" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G181" s="8"/>
     </row>
@@ -7386,7 +7390,7 @@
       </c>
       <c r="E182" s="11"/>
       <c r="F182" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G182" s="8"/>
     </row>
@@ -7405,7 +7409,7 @@
       </c>
       <c r="E183" s="11"/>
       <c r="F183" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G183" s="8"/>
     </row>
@@ -7424,7 +7428,7 @@
       </c>
       <c r="E184" s="11"/>
       <c r="F184" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G184" s="8"/>
     </row>
@@ -7443,7 +7447,7 @@
       </c>
       <c r="E185" s="11"/>
       <c r="F185" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G185" s="8"/>
     </row>
@@ -7462,7 +7466,7 @@
       </c>
       <c r="E186" s="11"/>
       <c r="F186" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G186" s="8"/>
     </row>
@@ -7481,7 +7485,7 @@
       </c>
       <c r="E187" s="11"/>
       <c r="F187" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G187" s="8"/>
     </row>
@@ -7500,7 +7504,7 @@
       </c>
       <c r="E188" s="11"/>
       <c r="F188" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G188" s="8"/>
     </row>
@@ -7519,7 +7523,7 @@
       </c>
       <c r="E189" s="11"/>
       <c r="F189" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G189" s="8"/>
     </row>
@@ -7538,7 +7542,7 @@
       </c>
       <c r="E190" s="11"/>
       <c r="F190" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G190" s="8"/>
     </row>
@@ -7557,7 +7561,7 @@
       </c>
       <c r="E191" s="11"/>
       <c r="F191" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G191" s="8"/>
     </row>
@@ -7577,7 +7581,9 @@
       <c r="E192" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="F192" s="8"/>
+      <c r="F192" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G192" s="8"/>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.25">
@@ -7594,7 +7600,9 @@
         <v>192</v>
       </c>
       <c r="E193" s="11"/>
-      <c r="F193" s="8"/>
+      <c r="F193" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G193" s="8"/>
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.25">
@@ -7611,7 +7619,9 @@
         <v>192</v>
       </c>
       <c r="E194" s="11"/>
-      <c r="F194" s="8"/>
+      <c r="F194" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G194" s="8"/>
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.25">
@@ -7628,7 +7638,9 @@
         <v>192</v>
       </c>
       <c r="E195" s="11"/>
-      <c r="F195" s="8"/>
+      <c r="F195" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G195" s="8"/>
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.25">
@@ -7645,7 +7657,9 @@
         <v>192</v>
       </c>
       <c r="E196" s="11"/>
-      <c r="F196" s="8"/>
+      <c r="F196" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G196" s="8"/>
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.25">
@@ -7662,7 +7676,9 @@
         <v>192</v>
       </c>
       <c r="E197" s="11"/>
-      <c r="F197" s="8"/>
+      <c r="F197" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G197" s="8"/>
     </row>
     <row r="198" spans="1:7" x14ac:dyDescent="0.25">
@@ -7679,7 +7695,9 @@
         <v>192</v>
       </c>
       <c r="E198" s="11"/>
-      <c r="F198" s="8"/>
+      <c r="F198" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G198" s="8"/>
     </row>
     <row r="199" spans="1:7" x14ac:dyDescent="0.25">
@@ -7696,7 +7714,9 @@
         <v>192</v>
       </c>
       <c r="E199" s="11"/>
-      <c r="F199" s="8"/>
+      <c r="F199" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G199" s="8"/>
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.25">
@@ -7713,7 +7733,9 @@
         <v>192</v>
       </c>
       <c r="E200" s="11"/>
-      <c r="F200" s="8"/>
+      <c r="F200" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G200" s="8"/>
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.25">
@@ -7730,7 +7752,9 @@
         <v>192</v>
       </c>
       <c r="E201" s="11"/>
-      <c r="F201" s="8"/>
+      <c r="F201" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G201" s="8"/>
     </row>
     <row r="202" spans="1:7" x14ac:dyDescent="0.25">
@@ -7747,7 +7771,9 @@
         <v>192</v>
       </c>
       <c r="E202" s="11"/>
-      <c r="F202" s="8"/>
+      <c r="F202" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G202" s="8"/>
     </row>
     <row r="203" spans="1:7" x14ac:dyDescent="0.25">
@@ -7764,7 +7790,9 @@
         <v>192</v>
       </c>
       <c r="E203" s="11"/>
-      <c r="F203" s="8"/>
+      <c r="F203" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G203" s="8"/>
     </row>
     <row r="204" spans="1:7" x14ac:dyDescent="0.25">
@@ -7781,7 +7809,9 @@
         <v>192</v>
       </c>
       <c r="E204" s="11"/>
-      <c r="F204" s="8"/>
+      <c r="F204" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G204" s="8"/>
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.25">
@@ -7798,7 +7828,9 @@
         <v>192</v>
       </c>
       <c r="E205" s="11"/>
-      <c r="F205" s="8"/>
+      <c r="F205" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G205" s="8"/>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.25">
@@ -7815,7 +7847,9 @@
         <v>192</v>
       </c>
       <c r="E206" s="11"/>
-      <c r="F206" s="8"/>
+      <c r="F206" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G206" s="8"/>
     </row>
     <row r="207" spans="1:7" x14ac:dyDescent="0.25">
@@ -7832,7 +7866,9 @@
         <v>192</v>
       </c>
       <c r="E207" s="11"/>
-      <c r="F207" s="8"/>
+      <c r="F207" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G207" s="8"/>
     </row>
     <row r="208" spans="1:7" x14ac:dyDescent="0.25">
@@ -7849,7 +7885,9 @@
         <v>192</v>
       </c>
       <c r="E208" s="11"/>
-      <c r="F208" s="8"/>
+      <c r="F208" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G208" s="8"/>
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.25">
@@ -7866,10 +7904,12 @@
         <v>192</v>
       </c>
       <c r="E209" s="11"/>
-      <c r="F209" s="8"/>
+      <c r="F209" s="8" t="s">
+        <v>224</v>
+      </c>
       <c r="G209" s="8"/>
     </row>
-    <row r="210" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="8" t="s">
         <v>42</v>
       </c>
@@ -7884,7 +7924,7 @@
       <c r="F210" s="8"/>
       <c r="G210" s="8"/>
     </row>
-    <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="8" t="s">
         <v>42</v>
       </c>
@@ -7899,7 +7939,7 @@
       <c r="F211" s="8"/>
       <c r="G211" s="8"/>
     </row>
-    <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" s="8" t="s">
         <v>42</v>
       </c>
@@ -7914,7 +7954,7 @@
       <c r="F212" s="8"/>
       <c r="G212" s="8"/>
     </row>
-    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" s="8" t="s">
         <v>42</v>
       </c>
@@ -7929,7 +7969,7 @@
       <c r="F213" s="8"/>
       <c r="G213" s="8"/>
     </row>
-    <row r="214" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="8" t="s">
         <v>42</v>
       </c>
@@ -7944,7 +7984,7 @@
       <c r="F214" s="8"/>
       <c r="G214" s="8"/>
     </row>
-    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" s="8" t="s">
         <v>42</v>
       </c>
@@ -7959,7 +7999,7 @@
       <c r="F215" s="8"/>
       <c r="G215" s="8"/>
     </row>
-    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="8" t="s">
         <v>42</v>
       </c>
@@ -7974,7 +8014,7 @@
       <c r="F216" s="8"/>
       <c r="G216" s="8"/>
     </row>
-    <row r="217" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="8" t="s">
         <v>42</v>
       </c>
@@ -7989,7 +8029,7 @@
       <c r="F217" s="8"/>
       <c r="G217" s="8"/>
     </row>
-    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="8" t="s">
         <v>42</v>
       </c>
@@ -8004,7 +8044,7 @@
       <c r="F218" s="8"/>
       <c r="G218" s="8"/>
     </row>
-    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="8" t="s">
         <v>42</v>
       </c>
@@ -8019,7 +8059,7 @@
       <c r="F219" s="8"/>
       <c r="G219" s="8"/>
     </row>
-    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="8" t="s">
         <v>42</v>
       </c>
@@ -8034,7 +8074,7 @@
       <c r="F220" s="8"/>
       <c r="G220" s="8"/>
     </row>
-    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
         <v>42</v>
       </c>
@@ -8049,7 +8089,7 @@
       <c r="F221" s="8"/>
       <c r="G221" s="8"/>
     </row>
-    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" s="8" t="s">
         <v>42</v>
       </c>
@@ -8064,7 +8104,7 @@
       <c r="F222" s="8"/>
       <c r="G222" s="8"/>
     </row>
-    <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="8" t="s">
         <v>42</v>
       </c>
@@ -8079,7 +8119,7 @@
       <c r="F223" s="8"/>
       <c r="G223" s="8"/>
     </row>
-    <row r="224" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" s="8" t="s">
         <v>42</v>
       </c>
@@ -8094,7 +8134,7 @@
       <c r="F224" s="8"/>
       <c r="G224" s="8"/>
     </row>
-    <row r="225" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" s="8" t="s">
         <v>42</v>
       </c>
@@ -8109,7 +8149,7 @@
       <c r="F225" s="8"/>
       <c r="G225" s="8"/>
     </row>
-    <row r="226" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" s="8" t="s">
         <v>42</v>
       </c>
@@ -8124,7 +8164,7 @@
       <c r="F226" s="8"/>
       <c r="G226" s="8"/>
     </row>
-    <row r="227" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" s="8" t="s">
         <v>42</v>
       </c>
@@ -8139,7 +8179,7 @@
       <c r="F227" s="8"/>
       <c r="G227" s="8"/>
     </row>
-    <row r="228" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" s="8" t="s">
         <v>42</v>
       </c>
@@ -8154,7 +8194,7 @@
       <c r="F228" s="8"/>
       <c r="G228" s="8"/>
     </row>
-    <row r="229" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" s="8" t="s">
         <v>42</v>
       </c>
@@ -8169,7 +8209,7 @@
       <c r="F229" s="8"/>
       <c r="G229" s="8"/>
     </row>
-    <row r="230" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230" s="8" t="s">
         <v>39</v>
       </c>
@@ -8184,7 +8224,7 @@
       <c r="F230" s="8"/>
       <c r="G230" s="8"/>
     </row>
-    <row r="231" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231" s="8" t="s">
         <v>39</v>
       </c>
@@ -8199,7 +8239,7 @@
       <c r="F231" s="8"/>
       <c r="G231" s="8"/>
     </row>
-    <row r="232" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232" s="8" t="s">
         <v>39</v>
       </c>
@@ -8214,7 +8254,7 @@
       <c r="F232" s="8"/>
       <c r="G232" s="8"/>
     </row>
-    <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" s="8" t="s">
         <v>39</v>
       </c>
@@ -8229,7 +8269,7 @@
       <c r="F233" s="8"/>
       <c r="G233" s="8"/>
     </row>
-    <row r="234" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234" s="8" t="s">
         <v>39</v>
       </c>
@@ -8244,7 +8284,7 @@
       <c r="F234" s="8"/>
       <c r="G234" s="8"/>
     </row>
-    <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" s="8" t="s">
         <v>39</v>
       </c>
@@ -8259,7 +8299,7 @@
       <c r="F235" s="8"/>
       <c r="G235" s="8"/>
     </row>
-    <row r="236" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236" s="8" t="s">
         <v>39</v>
       </c>
@@ -8274,7 +8314,7 @@
       <c r="F236" s="8"/>
       <c r="G236" s="8"/>
     </row>
-    <row r="237" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" s="8" t="s">
         <v>39</v>
       </c>
@@ -8289,7 +8329,7 @@
       <c r="F237" s="8"/>
       <c r="G237" s="8"/>
     </row>
-    <row r="238" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" s="8" t="s">
         <v>39</v>
       </c>
@@ -8304,7 +8344,7 @@
       <c r="F238" s="8"/>
       <c r="G238" s="8"/>
     </row>
-    <row r="239" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239" s="8" t="s">
         <v>39</v>
       </c>
@@ -8319,7 +8359,7 @@
       <c r="F239" s="8"/>
       <c r="G239" s="8"/>
     </row>
-    <row r="240" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A240" s="8" t="s">
         <v>41</v>
       </c>
@@ -8338,7 +8378,7 @@
       <c r="F240" s="8"/>
       <c r="G240" s="8"/>
     </row>
-    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A241" s="8" t="s">
         <v>41</v>
       </c>
@@ -8355,7 +8395,7 @@
       <c r="F241" s="8"/>
       <c r="G241" s="8"/>
     </row>
-    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242" s="8" t="s">
         <v>41</v>
       </c>
@@ -8372,7 +8412,7 @@
       <c r="F242" s="8"/>
       <c r="G242" s="8"/>
     </row>
-    <row r="243" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243" s="8" t="s">
         <v>41</v>
       </c>
@@ -8389,7 +8429,7 @@
       <c r="F243" s="8"/>
       <c r="G243" s="8"/>
     </row>
-    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244" s="8" t="s">
         <v>41</v>
       </c>
@@ -8406,7 +8446,7 @@
       <c r="F244" s="8"/>
       <c r="G244" s="8"/>
     </row>
-    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A245" s="8" t="s">
         <v>41</v>
       </c>
@@ -8423,7 +8463,7 @@
       <c r="F245" s="8"/>
       <c r="G245" s="8"/>
     </row>
-    <row r="246" spans="1:7" ht="52.8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A246" s="8" t="s">
         <v>41</v>
       </c>
@@ -8442,7 +8482,7 @@
       <c r="F246" s="8"/>
       <c r="G246" s="8"/>
     </row>
-    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247" s="8" t="s">
         <v>41</v>
       </c>
@@ -8459,7 +8499,7 @@
       <c r="F247" s="8"/>
       <c r="G247" s="8"/>
     </row>
-    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248" s="8" t="s">
         <v>41</v>
       </c>
@@ -8476,7 +8516,7 @@
       <c r="F248" s="8"/>
       <c r="G248" s="8"/>
     </row>
-    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A249" s="8" t="s">
         <v>41</v>
       </c>
@@ -8493,7 +8533,7 @@
       <c r="F249" s="8"/>
       <c r="G249" s="8"/>
     </row>
-    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250" s="8" t="s">
         <v>41</v>
       </c>
@@ -8510,7 +8550,7 @@
       <c r="F250" s="8"/>
       <c r="G250" s="8"/>
     </row>
-    <row r="251" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251" s="8" t="s">
         <v>41</v>
       </c>
@@ -8527,7 +8567,7 @@
       <c r="F251" s="8"/>
       <c r="G251" s="8"/>
     </row>
-    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A252" s="8" t="s">
         <v>41</v>
       </c>
@@ -8544,7 +8584,7 @@
       <c r="F252" s="8"/>
       <c r="G252" s="8"/>
     </row>
-    <row r="253" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253" s="8" t="s">
         <v>41</v>
       </c>
@@ -8561,7 +8601,7 @@
       <c r="F253" s="8"/>
       <c r="G253" s="8"/>
     </row>
-    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A254" s="8" t="s">
         <v>41</v>
       </c>
@@ -8578,7 +8618,7 @@
       <c r="F254" s="8"/>
       <c r="G254" s="8"/>
     </row>
-    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" s="8" t="s">
         <v>41</v>
       </c>
@@ -8595,7 +8635,7 @@
       <c r="F255" s="8"/>
       <c r="G255" s="8"/>
     </row>
-    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A256" s="8" t="s">
         <v>41</v>
       </c>
@@ -8612,7 +8652,7 @@
       <c r="F256" s="8"/>
       <c r="G256" s="8"/>
     </row>
-    <row r="257" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A257" s="8" t="s">
         <v>41</v>
       </c>
@@ -8629,7 +8669,7 @@
       <c r="F257" s="8"/>
       <c r="G257" s="8"/>
     </row>
-    <row r="258" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A258" s="8" t="s">
         <v>41</v>
       </c>
@@ -8646,7 +8686,7 @@
       <c r="F258" s="8"/>
       <c r="G258" s="8"/>
     </row>
-    <row r="259" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A259" s="8" t="s">
         <v>41</v>
       </c>
@@ -8663,7 +8703,7 @@
       <c r="F259" s="8"/>
       <c r="G259" s="8"/>
     </row>
-    <row r="260" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A260" s="8" t="s">
         <v>41</v>
       </c>
@@ -8680,7 +8720,7 @@
       <c r="F260" s="8"/>
       <c r="G260" s="8"/>
     </row>
-    <row r="261" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A261" s="8" t="s">
         <v>41</v>
       </c>
@@ -8697,7 +8737,7 @@
       <c r="F261" s="8"/>
       <c r="G261" s="8"/>
     </row>
-    <row r="262" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A262" s="8" t="s">
         <v>41</v>
       </c>
@@ -8714,7 +8754,7 @@
       <c r="F262" s="8"/>
       <c r="G262" s="8"/>
     </row>
-    <row r="263" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A263" s="8" t="s">
         <v>41</v>
       </c>
@@ -8731,7 +8771,7 @@
       <c r="F263" s="8"/>
       <c r="G263" s="8"/>
     </row>
-    <row r="264" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A264" s="8" t="s">
         <v>41</v>
       </c>
@@ -8748,7 +8788,7 @@
       <c r="F264" s="8"/>
       <c r="G264" s="8"/>
     </row>
-    <row r="265" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A265" s="8" t="s">
         <v>41</v>
       </c>
@@ -8765,7 +8805,7 @@
       <c r="F265" s="8"/>
       <c r="G265" s="8"/>
     </row>
-    <row r="266" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A266" s="8" t="s">
         <v>41</v>
       </c>
@@ -8782,7 +8822,7 @@
       <c r="F266" s="8"/>
       <c r="G266" s="8"/>
     </row>
-    <row r="267" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A267" s="8" t="s">
         <v>41</v>
       </c>
@@ -8799,7 +8839,7 @@
       <c r="F267" s="8"/>
       <c r="G267" s="8"/>
     </row>
-    <row r="268" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A268" s="8" t="s">
         <v>41</v>
       </c>
@@ -8816,7 +8856,7 @@
       <c r="F268" s="8"/>
       <c r="G268" s="8"/>
     </row>
-    <row r="269" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A269" s="8" t="s">
         <v>41</v>
       </c>
@@ -8833,7 +8873,7 @@
       <c r="F269" s="8"/>
       <c r="G269" s="8"/>
     </row>
-    <row r="270" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A270" s="8" t="s">
         <v>41</v>
       </c>
@@ -8850,7 +8890,7 @@
       <c r="F270" s="8"/>
       <c r="G270" s="8"/>
     </row>
-    <row r="271" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A271" s="8" t="s">
         <v>41</v>
       </c>
@@ -8867,7 +8907,7 @@
       <c r="F271" s="8"/>
       <c r="G271" s="8"/>
     </row>
-    <row r="272" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A272" s="8" t="s">
         <v>41</v>
       </c>
@@ -8884,7 +8924,7 @@
       <c r="F272" s="8"/>
       <c r="G272" s="8"/>
     </row>
-    <row r="273" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A273" s="8" t="s">
         <v>41</v>
       </c>
@@ -8901,7 +8941,7 @@
       <c r="F273" s="8"/>
       <c r="G273" s="8"/>
     </row>
-    <row r="274" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A274" s="8" t="s">
         <v>41</v>
       </c>
@@ -8918,7 +8958,7 @@
       <c r="F274" s="8"/>
       <c r="G274" s="8"/>
     </row>
-    <row r="275" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A275" s="8" t="s">
         <v>41</v>
       </c>
@@ -8935,7 +8975,7 @@
       <c r="F275" s="8"/>
       <c r="G275" s="8"/>
     </row>
-    <row r="276" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A276" s="8" t="s">
         <v>41</v>
       </c>
@@ -8952,7 +8992,7 @@
       <c r="F276" s="8"/>
       <c r="G276" s="8"/>
     </row>
-    <row r="277" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A277" s="8" t="s">
         <v>41</v>
       </c>
@@ -8969,7 +9009,7 @@
       <c r="F277" s="8"/>
       <c r="G277" s="8"/>
     </row>
-    <row r="278" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A278" s="8" t="s">
         <v>41</v>
       </c>
@@ -8986,7 +9026,7 @@
       <c r="F278" s="8"/>
       <c r="G278" s="8"/>
     </row>
-    <row r="279" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A279" s="8" t="s">
         <v>41</v>
       </c>
@@ -9005,7 +9045,7 @@
       <c r="F279" s="8"/>
       <c r="G279" s="8"/>
     </row>
-    <row r="280" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A280" s="8" t="s">
         <v>41</v>
       </c>
@@ -9022,7 +9062,7 @@
       <c r="F280" s="8"/>
       <c r="G280" s="8"/>
     </row>
-    <row r="281" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A281" s="8" t="s">
         <v>41</v>
       </c>
@@ -9039,7 +9079,7 @@
       <c r="F281" s="8"/>
       <c r="G281" s="8"/>
     </row>
-    <row r="282" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A282" s="8" t="s">
         <v>41</v>
       </c>
@@ -9056,7 +9096,7 @@
       <c r="F282" s="8"/>
       <c r="G282" s="8"/>
     </row>
-    <row r="283" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A283" s="8" t="s">
         <v>41</v>
       </c>
@@ -9073,7 +9113,7 @@
       <c r="F283" s="8"/>
       <c r="G283" s="8"/>
     </row>
-    <row r="284" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A284" s="8" t="s">
         <v>41</v>
       </c>
@@ -9090,7 +9130,7 @@
       <c r="F284" s="8"/>
       <c r="G284" s="8"/>
     </row>
-    <row r="285" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A285" s="8" t="s">
         <v>41</v>
       </c>
@@ -9107,7 +9147,7 @@
       <c r="F285" s="8"/>
       <c r="G285" s="8"/>
     </row>
-    <row r="286" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A286" s="8" t="s">
         <v>41</v>
       </c>
@@ -9124,7 +9164,7 @@
       <c r="F286" s="8"/>
       <c r="G286" s="8"/>
     </row>
-    <row r="287" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A287" s="8" t="s">
         <v>41</v>
       </c>
@@ -9141,7 +9181,7 @@
       <c r="F287" s="8"/>
       <c r="G287" s="8"/>
     </row>
-    <row r="288" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A288" s="8" t="s">
         <v>41</v>
       </c>
@@ -9158,7 +9198,7 @@
       <c r="F288" s="8"/>
       <c r="G288" s="8"/>
     </row>
-    <row r="289" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A289" s="8" t="s">
         <v>41</v>
       </c>
@@ -9175,7 +9215,7 @@
       <c r="F289" s="8"/>
       <c r="G289" s="8"/>
     </row>
-    <row r="290" spans="1:7" ht="39.6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A290" s="8" t="s">
         <v>41</v>
       </c>
@@ -9194,7 +9234,7 @@
       <c r="F290" s="8"/>
       <c r="G290" s="8"/>
     </row>
-    <row r="291" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A291" s="8" t="s">
         <v>41</v>
       </c>
@@ -9211,7 +9251,7 @@
       <c r="F291" s="8"/>
       <c r="G291" s="8"/>
     </row>
-    <row r="292" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A292" s="8" t="s">
         <v>41</v>
       </c>
@@ -9228,7 +9268,7 @@
       <c r="F292" s="8"/>
       <c r="G292" s="8"/>
     </row>
-    <row r="293" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A293" s="8" t="s">
         <v>41</v>
       </c>
@@ -9245,7 +9285,7 @@
       <c r="F293" s="8"/>
       <c r="G293" s="8"/>
     </row>
-    <row r="294" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A294" s="8" t="s">
         <v>41</v>
       </c>
@@ -9262,7 +9302,7 @@
       <c r="F294" s="8"/>
       <c r="G294" s="8"/>
     </row>
-    <row r="295" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A295" s="8" t="s">
         <v>41</v>
       </c>
@@ -9279,7 +9319,7 @@
       <c r="F295" s="8"/>
       <c r="G295" s="8"/>
     </row>
-    <row r="296" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A296" s="8" t="s">
         <v>41</v>
       </c>
@@ -9296,7 +9336,7 @@
       <c r="F296" s="8"/>
       <c r="G296" s="8"/>
     </row>
-    <row r="297" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A297" s="8" t="s">
         <v>41</v>
       </c>
@@ -9313,7 +9353,7 @@
       <c r="F297" s="8"/>
       <c r="G297" s="8"/>
     </row>
-    <row r="298" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A298" s="8" t="s">
         <v>41</v>
       </c>
@@ -9330,7 +9370,7 @@
       <c r="F298" s="8"/>
       <c r="G298" s="8"/>
     </row>
-    <row r="299" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A299" s="8" t="s">
         <v>41</v>
       </c>
@@ -9347,7 +9387,7 @@
       <c r="F299" s="8"/>
       <c r="G299" s="8"/>
     </row>
-    <row r="300" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A300" s="8" t="s">
         <v>41</v>
       </c>
@@ -9366,16 +9406,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G300" xr:uid="{38A162FC-7907-44C7-A909-E8E1323EC5F6}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="seabream"/>
-      </filters>
-    </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:G20">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A240:G300">
       <sortCondition ref="D1:D300"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="G2 F5:G5 F2:F300">
+  <conditionalFormatting sqref="G2 F2:F300 F5:G5">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>

</xml_diff>